<commit_message>
EBS pollock: drop double-counted Japanese CPUE
The base xlsx attaches the 1965-1976 Japanese CPUE to the Fishery fleet
(Fleet_code 1) as an index, and data.R re-adds the same 12 observations as
a dedicated CPUE survey fleet (mirroring the fishery selectivity with its own
estimated q, matching ADMB's single cpue_like). Leaving the base copy fit the
CPUE twice; since those obs are the only early-period index (1965-1976), the
double-count over-constrained the initial age structure and pulled the early
years off ADMB. Drop the base fishery-index rows so the CPUE is fit once.
</commit_message>
<xml_diff>
--- a/EBS pollock/Data/2024_EBS_pollock_m23_rceattle_full.xlsx
+++ b/EBS pollock/Data/2024_EBS_pollock_m23_rceattle_full.xlsx
@@ -35553,7 +35553,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I165"/>
+  <dimension ref="A1:I153"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -35606,17 +35606,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Fishery CPUE</t>
+          <t>AVO</t>
         </is>
       </c>
       <c r="B2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C2">
         <v>1</v>
       </c>
       <c r="D2">
-        <v>1965</v>
+        <v>2006</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -35628,26 +35628,26 @@
         <v>1</v>
       </c>
       <c r="H2">
-        <v>2816.437428</v>
+        <v>1.741476103</v>
       </c>
       <c r="I2">
-        <v>0.2</v>
+        <v>0.407974331</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Fishery CPUE</t>
+          <t>AVO</t>
         </is>
       </c>
       <c r="B3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C3">
         <v>1</v>
       </c>
       <c r="D3">
-        <v>1966</v>
+        <v>2007</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -35659,26 +35659,26 @@
         <v>1</v>
       </c>
       <c r="H3">
-        <v>3473.580475</v>
+        <v>2.00191307</v>
       </c>
       <c r="I3">
-        <v>0.2</v>
+        <v>0.79543824</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Fishery CPUE</t>
+          <t>AVO</t>
         </is>
       </c>
       <c r="B4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C4">
         <v>1</v>
       </c>
       <c r="D4">
-        <v>1967</v>
+        <v>2008</v>
       </c>
       <c r="E4">
         <v>0</v>
@@ -35690,26 +35690,26 @@
         <v>1</v>
       </c>
       <c r="H4">
-        <v>3802.169891</v>
+        <v>0.991543151</v>
       </c>
       <c r="I4">
-        <v>0.1999999999736992</v>
+        <v>0.292865177</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Fishery CPUE</t>
+          <t>AVO</t>
         </is>
       </c>
       <c r="B5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C5">
         <v>1</v>
       </c>
       <c r="D5">
-        <v>1968</v>
+        <v>2009</v>
       </c>
       <c r="E5">
         <v>0</v>
@@ -35721,26 +35721,26 @@
         <v>1</v>
       </c>
       <c r="H5">
-        <v>5257.304601</v>
+        <v>0.6951000000000001</v>
       </c>
       <c r="I5">
-        <v>0.1999999999619577</v>
+        <v>0.390095688</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Fishery CPUE</t>
+          <t>AVO</t>
         </is>
       </c>
       <c r="B6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C6">
         <v>1</v>
       </c>
       <c r="D6">
-        <v>1969</v>
+        <v>2010</v>
       </c>
       <c r="E6">
         <v>0</v>
@@ -35752,26 +35752,26 @@
         <v>1</v>
       </c>
       <c r="H6">
-        <v>6712.468418</v>
+        <v>1.9218</v>
       </c>
       <c r="I6">
-        <v>0.2000000000595906</v>
+        <v>0.579193251</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Fishery CPUE</t>
+          <t>AVO</t>
         </is>
       </c>
       <c r="B7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C7">
         <v>1</v>
       </c>
       <c r="D7">
-        <v>1970</v>
+        <v>2011</v>
       </c>
       <c r="E7">
         <v>0</v>
@@ -35783,26 +35783,26 @@
         <v>1</v>
       </c>
       <c r="H7">
-        <v>5679.809828</v>
+        <v>1.703822566</v>
       </c>
       <c r="I7">
-        <v>0.2000000000704249</v>
+        <v>0.447677778</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Fishery CPUE</t>
+          <t>AVO</t>
         </is>
       </c>
       <c r="B8">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C8">
         <v>1</v>
       </c>
       <c r="D8">
-        <v>1971</v>
+        <v>2012</v>
       </c>
       <c r="E8">
         <v>0</v>
@@ -35814,26 +35814,26 @@
         <v>1</v>
       </c>
       <c r="H8">
-        <v>5257.331283</v>
+        <v>1.5206</v>
       </c>
       <c r="I8">
-        <v>0.2000000000760842</v>
+        <v>0.371938445</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Fishery CPUE</t>
+          <t>AVO</t>
         </is>
       </c>
       <c r="B9">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C9">
         <v>1</v>
       </c>
       <c r="D9">
-        <v>1972</v>
+        <v>2013</v>
       </c>
       <c r="E9">
         <v>0</v>
@@ -35845,26 +35845,26 @@
         <v>1</v>
       </c>
       <c r="H9">
-        <v>5726.743484</v>
+        <v>2.177629578</v>
       </c>
       <c r="I9">
-        <v>0.2000000000349239</v>
+        <v>0.390115995</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Fishery CPUE</t>
+          <t>AVO</t>
         </is>
       </c>
       <c r="B10">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C10">
         <v>1</v>
       </c>
       <c r="D10">
-        <v>1973</v>
+        <v>2014</v>
       </c>
       <c r="E10">
         <v>0</v>
@@ -35876,26 +35876,26 @@
         <v>1</v>
       </c>
       <c r="H10">
-        <v>4787.923949</v>
+        <v>3.0769</v>
       </c>
       <c r="I10">
-        <v>0.2</v>
+        <v>0.5802458700000001</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Fishery CPUE</t>
+          <t>AVO</t>
         </is>
       </c>
       <c r="B11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C11">
         <v>1</v>
       </c>
       <c r="D11">
-        <v>1974</v>
+        <v>2015</v>
       </c>
       <c r="E11">
         <v>0</v>
@@ -35907,26 +35907,26 @@
         <v>1</v>
       </c>
       <c r="H11">
-        <v>4740.992588</v>
+        <v>3.5927</v>
       </c>
       <c r="I11">
-        <v>0.2</v>
+        <v>0.406257388</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Fishery CPUE</t>
+          <t>AVO</t>
         </is>
       </c>
       <c r="B12">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C12">
         <v>1</v>
       </c>
       <c r="D12">
-        <v>1975</v>
+        <v>2016</v>
       </c>
       <c r="E12">
         <v>0</v>
@@ -35938,26 +35938,26 @@
         <v>1</v>
       </c>
       <c r="H12">
-        <v>4271.57446</v>
+        <v>2.8319</v>
       </c>
       <c r="I12">
-        <v>0.1999999999765894</v>
+        <v>0.379092753</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Fishery CPUE</t>
+          <t>AVO</t>
         </is>
       </c>
       <c r="B13">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C13">
         <v>1</v>
       </c>
       <c r="D13">
-        <v>1976</v>
+        <v>2017</v>
       </c>
       <c r="E13">
         <v>0</v>
@@ -35969,10 +35969,10 @@
         <v>1</v>
       </c>
       <c r="H13">
-        <v>4318.523058</v>
+        <v>2.263</v>
       </c>
       <c r="I13">
-        <v>0.2</v>
+        <v>0.317389245</v>
       </c>
     </row>
     <row r="14">
@@ -35988,7 +35988,7 @@
         <v>1</v>
       </c>
       <c r="D14">
-        <v>2006</v>
+        <v>2018</v>
       </c>
       <c r="E14">
         <v>0</v>
@@ -36000,10 +36000,10 @@
         <v>1</v>
       </c>
       <c r="H14">
-        <v>1.741476103</v>
+        <v>2.0841</v>
       </c>
       <c r="I14">
-        <v>0.407974331</v>
+        <v>0.254960502</v>
       </c>
     </row>
     <row r="15">
@@ -36019,7 +36019,7 @@
         <v>1</v>
       </c>
       <c r="D15">
-        <v>2007</v>
+        <v>2019</v>
       </c>
       <c r="E15">
         <v>0</v>
@@ -36031,10 +36031,10 @@
         <v>1</v>
       </c>
       <c r="H15">
-        <v>2.00191307</v>
+        <v>2.8292</v>
       </c>
       <c r="I15">
-        <v>0.79543824</v>
+        <v>0.63539506</v>
       </c>
     </row>
     <row r="16">
@@ -36050,7 +36050,7 @@
         <v>1</v>
       </c>
       <c r="D16">
-        <v>2008</v>
+        <v>2021</v>
       </c>
       <c r="E16">
         <v>0</v>
@@ -36062,10 +36062,10 @@
         <v>1</v>
       </c>
       <c r="H16">
-        <v>0.991543151</v>
+        <v>2.4101</v>
       </c>
       <c r="I16">
-        <v>0.292865177</v>
+        <v>0.529928784</v>
       </c>
     </row>
     <row r="17">
@@ -36081,7 +36081,7 @@
         <v>1</v>
       </c>
       <c r="D17">
-        <v>2009</v>
+        <v>2022</v>
       </c>
       <c r="E17">
         <v>0</v>
@@ -36093,10 +36093,10 @@
         <v>1</v>
       </c>
       <c r="H17">
-        <v>0.6951000000000001</v>
+        <v>2.9031</v>
       </c>
       <c r="I17">
-        <v>0.390095688</v>
+        <v>0.454780316</v>
       </c>
     </row>
     <row r="18">
@@ -36112,7 +36112,7 @@
         <v>1</v>
       </c>
       <c r="D18">
-        <v>2010</v>
+        <v>2023</v>
       </c>
       <c r="E18">
         <v>0</v>
@@ -36124,10 +36124,10 @@
         <v>1</v>
       </c>
       <c r="H18">
-        <v>1.9218</v>
+        <v>2.481</v>
       </c>
       <c r="I18">
-        <v>0.579193251</v>
+        <v>0.335349192</v>
       </c>
     </row>
     <row r="19">
@@ -36143,7 +36143,7 @@
         <v>1</v>
       </c>
       <c r="D19">
-        <v>2011</v>
+        <v>2024</v>
       </c>
       <c r="E19">
         <v>0</v>
@@ -36155,29 +36155,29 @@
         <v>1</v>
       </c>
       <c r="H19">
-        <v>1.703822566</v>
+        <v>2.00700959</v>
       </c>
       <c r="I19">
-        <v>0.447677778</v>
+        <v>0.250814465</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>AVO</t>
+          <t>BTS</t>
         </is>
       </c>
       <c r="B20">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C20">
         <v>1</v>
       </c>
       <c r="D20">
-        <v>2012</v>
+        <v>1982</v>
       </c>
       <c r="E20">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="F20">
         <v>1</v>
@@ -36186,29 +36186,29 @@
         <v>1</v>
       </c>
       <c r="H20">
-        <v>1.5206</v>
+        <v>3871.045939</v>
       </c>
       <c r="I20">
-        <v>0.371938445</v>
+        <v>0.0726252533630808</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>AVO</t>
+          <t>BTS</t>
         </is>
       </c>
       <c r="B21">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C21">
         <v>1</v>
       </c>
       <c r="D21">
-        <v>2013</v>
+        <v>1983</v>
       </c>
       <c r="E21">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="F21">
         <v>1</v>
@@ -36217,29 +36217,29 @@
         <v>1</v>
       </c>
       <c r="H21">
-        <v>2.177629578</v>
+        <v>8918.551101999999</v>
       </c>
       <c r="I21">
-        <v>0.390115995</v>
+        <v>0.06436800069141994</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>AVO</t>
+          <t>BTS</t>
         </is>
       </c>
       <c r="B22">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C22">
         <v>1</v>
       </c>
       <c r="D22">
-        <v>2014</v>
+        <v>1984</v>
       </c>
       <c r="E22">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="F22">
         <v>1</v>
@@ -36248,29 +36248,29 @@
         <v>1</v>
       </c>
       <c r="H22">
-        <v>3.0769</v>
+        <v>6575.015167</v>
       </c>
       <c r="I22">
-        <v>0.5802458700000001</v>
+        <v>0.06670849626345812</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>AVO</t>
+          <t>BTS</t>
         </is>
       </c>
       <c r="B23">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C23">
         <v>1</v>
       </c>
       <c r="D23">
-        <v>2015</v>
+        <v>1985</v>
       </c>
       <c r="E23">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="F23">
         <v>1</v>
@@ -36279,29 +36279,29 @@
         <v>1</v>
       </c>
       <c r="H23">
-        <v>3.5927</v>
+        <v>7504.611645</v>
       </c>
       <c r="I23">
-        <v>0.406257388</v>
+        <v>0.07425474357107789</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>AVO</t>
+          <t>BTS</t>
         </is>
       </c>
       <c r="B24">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C24">
         <v>1</v>
       </c>
       <c r="D24">
-        <v>2016</v>
+        <v>1986</v>
       </c>
       <c r="E24">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="F24">
         <v>1</v>
@@ -36310,29 +36310,29 @@
         <v>1</v>
       </c>
       <c r="H24">
-        <v>2.8319</v>
+        <v>7235.877523</v>
       </c>
       <c r="I24">
-        <v>0.379092753</v>
+        <v>0.07273833548550514</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>AVO</t>
+          <t>BTS</t>
         </is>
       </c>
       <c r="B25">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C25">
         <v>1</v>
       </c>
       <c r="D25">
-        <v>2017</v>
+        <v>1987</v>
       </c>
       <c r="E25">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="F25">
         <v>1</v>
@@ -36341,29 +36341,29 @@
         <v>1</v>
       </c>
       <c r="H25">
-        <v>2.263</v>
+        <v>7576.038971</v>
       </c>
       <c r="I25">
-        <v>0.317389245</v>
+        <v>0.07848028377044103</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>AVO</t>
+          <t>BTS</t>
         </is>
       </c>
       <c r="B26">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C26">
         <v>1</v>
       </c>
       <c r="D26">
-        <v>2018</v>
+        <v>1988</v>
       </c>
       <c r="E26">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="F26">
         <v>1</v>
@@ -36372,29 +36372,29 @@
         <v>1</v>
       </c>
       <c r="H26">
-        <v>2.0841</v>
+        <v>11799.52504</v>
       </c>
       <c r="I26">
-        <v>0.254960502</v>
+        <v>0.08184918667709357</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>AVO</t>
+          <t>BTS</t>
         </is>
       </c>
       <c r="B27">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C27">
         <v>1</v>
       </c>
       <c r="D27">
-        <v>2019</v>
+        <v>1989</v>
       </c>
       <c r="E27">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="F27">
         <v>1</v>
@@ -36403,29 +36403,29 @@
         <v>1</v>
       </c>
       <c r="H27">
-        <v>2.8292</v>
+        <v>9942.601905</v>
       </c>
       <c r="I27">
-        <v>0.63539506</v>
+        <v>0.07006432365050022</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>AVO</t>
+          <t>BTS</t>
         </is>
       </c>
       <c r="B28">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C28">
         <v>1</v>
       </c>
       <c r="D28">
-        <v>2021</v>
+        <v>1990</v>
       </c>
       <c r="E28">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="F28">
         <v>1</v>
@@ -36434,29 +36434,29 @@
         <v>1</v>
       </c>
       <c r="H28">
-        <v>2.4101</v>
+        <v>11581.25353</v>
       </c>
       <c r="I28">
-        <v>0.529928784</v>
+        <v>0.08549051219155894</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>AVO</t>
+          <t>BTS</t>
         </is>
       </c>
       <c r="B29">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C29">
         <v>1</v>
       </c>
       <c r="D29">
-        <v>2022</v>
+        <v>1991</v>
       </c>
       <c r="E29">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="F29">
         <v>1</v>
@@ -36465,29 +36465,29 @@
         <v>1</v>
       </c>
       <c r="H29">
-        <v>2.9031</v>
+        <v>7129.587182</v>
       </c>
       <c r="I29">
-        <v>0.454780316</v>
+        <v>0.06822543938140738</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>AVO</t>
+          <t>BTS</t>
         </is>
       </c>
       <c r="B30">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C30">
         <v>1</v>
       </c>
       <c r="D30">
-        <v>2023</v>
+        <v>1992</v>
       </c>
       <c r="E30">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="F30">
         <v>1</v>
@@ -36496,29 +36496,29 @@
         <v>1</v>
       </c>
       <c r="H30">
-        <v>2.481</v>
+        <v>6643.437096</v>
       </c>
       <c r="I30">
-        <v>0.335349192</v>
+        <v>0.06902181079972704</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>AVO</t>
+          <t>BTS</t>
         </is>
       </c>
       <c r="B31">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C31">
         <v>1</v>
       </c>
       <c r="D31">
-        <v>2024</v>
+        <v>1993</v>
       </c>
       <c r="E31">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="F31">
         <v>1</v>
@@ -36527,10 +36527,10 @@
         <v>1</v>
       </c>
       <c r="H31">
-        <v>2.00700959</v>
+        <v>7849.269927</v>
       </c>
       <c r="I31">
-        <v>0.250814465</v>
+        <v>0.06360506917753753</v>
       </c>
     </row>
     <row r="32">
@@ -36546,7 +36546,7 @@
         <v>1</v>
       </c>
       <c r="D32">
-        <v>1982</v>
+        <v>1994</v>
       </c>
       <c r="E32">
         <v>6</v>
@@ -36558,10 +36558,10 @@
         <v>1</v>
       </c>
       <c r="H32">
-        <v>3871.045939</v>
+        <v>7094.434902</v>
       </c>
       <c r="I32">
-        <v>0.0726252533630808</v>
+        <v>0.06544262343842422</v>
       </c>
     </row>
     <row r="33">
@@ -36577,7 +36577,7 @@
         <v>1</v>
       </c>
       <c r="D33">
-        <v>1983</v>
+        <v>1995</v>
       </c>
       <c r="E33">
         <v>6</v>
@@ -36589,10 +36589,10 @@
         <v>1</v>
       </c>
       <c r="H33">
-        <v>8918.551101999999</v>
+        <v>6597.187752</v>
       </c>
       <c r="I33">
-        <v>0.06436800069141994</v>
+        <v>0.08288083056818238</v>
       </c>
     </row>
     <row r="34">
@@ -36608,7 +36608,7 @@
         <v>1</v>
       </c>
       <c r="D34">
-        <v>1984</v>
+        <v>1996</v>
       </c>
       <c r="E34">
         <v>6</v>
@@ -36620,10 +36620,10 @@
         <v>1</v>
       </c>
       <c r="H34">
-        <v>6575.015167</v>
+        <v>3954.25528</v>
       </c>
       <c r="I34">
-        <v>0.06670849626345812</v>
+        <v>0.06123113690322998</v>
       </c>
     </row>
     <row r="35">
@@ -36639,7 +36639,7 @@
         <v>1</v>
       </c>
       <c r="D35">
-        <v>1985</v>
+        <v>1997</v>
       </c>
       <c r="E35">
         <v>6</v>
@@ -36651,10 +36651,10 @@
         <v>1</v>
       </c>
       <c r="H35">
-        <v>7504.611645</v>
+        <v>4371.517782</v>
       </c>
       <c r="I35">
-        <v>0.07425474357107789</v>
+        <v>0.062961542929851</v>
       </c>
     </row>
     <row r="36">
@@ -36670,7 +36670,7 @@
         <v>1</v>
       </c>
       <c r="D36">
-        <v>1986</v>
+        <v>1998</v>
       </c>
       <c r="E36">
         <v>6</v>
@@ -36682,10 +36682,10 @@
         <v>1</v>
       </c>
       <c r="H36">
-        <v>7235.877523</v>
+        <v>3417.606809</v>
       </c>
       <c r="I36">
-        <v>0.07273833548550514</v>
+        <v>0.06118056598827428</v>
       </c>
     </row>
     <row r="37">
@@ -36701,7 +36701,7 @@
         <v>1</v>
       </c>
       <c r="D37">
-        <v>1987</v>
+        <v>1999</v>
       </c>
       <c r="E37">
         <v>6</v>
@@ -36713,10 +36713,10 @@
         <v>1</v>
       </c>
       <c r="H37">
-        <v>7576.038971</v>
+        <v>5613.644193</v>
       </c>
       <c r="I37">
-        <v>0.07848028377044103</v>
+        <v>0.07159299908981602</v>
       </c>
     </row>
     <row r="38">
@@ -36732,7 +36732,7 @@
         <v>1</v>
       </c>
       <c r="D38">
-        <v>1988</v>
+        <v>2000</v>
       </c>
       <c r="E38">
         <v>6</v>
@@ -36744,10 +36744,10 @@
         <v>1</v>
       </c>
       <c r="H38">
-        <v>11799.52504</v>
+        <v>7246.347745</v>
       </c>
       <c r="I38">
-        <v>0.08184918667709357</v>
+        <v>0.07060087017670444</v>
       </c>
     </row>
     <row r="39">
@@ -36763,7 +36763,7 @@
         <v>1</v>
       </c>
       <c r="D39">
-        <v>1989</v>
+        <v>2001</v>
       </c>
       <c r="E39">
         <v>6</v>
@@ -36775,10 +36775,10 @@
         <v>1</v>
       </c>
       <c r="H39">
-        <v>9942.601905</v>
+        <v>6066.56982</v>
       </c>
       <c r="I39">
-        <v>0.07006432365050022</v>
+        <v>0.06576865219363782</v>
       </c>
     </row>
     <row r="40">
@@ -36794,7 +36794,7 @@
         <v>1</v>
       </c>
       <c r="D40">
-        <v>1990</v>
+        <v>2002</v>
       </c>
       <c r="E40">
         <v>6</v>
@@ -36806,10 +36806,10 @@
         <v>1</v>
       </c>
       <c r="H40">
-        <v>11581.25353</v>
+        <v>6740.603163</v>
       </c>
       <c r="I40">
-        <v>0.08549051219155894</v>
+        <v>0.05824869705358147</v>
       </c>
     </row>
     <row r="41">
@@ -36825,7 +36825,7 @@
         <v>1</v>
       </c>
       <c r="D41">
-        <v>1991</v>
+        <v>2003</v>
       </c>
       <c r="E41">
         <v>6</v>
@@ -36837,10 +36837,10 @@
         <v>1</v>
       </c>
       <c r="H41">
-        <v>7129.587182</v>
+        <v>11239.16293</v>
       </c>
       <c r="I41">
-        <v>0.06822543938140738</v>
+        <v>0.06842173667109566</v>
       </c>
     </row>
     <row r="42">
@@ -36856,7 +36856,7 @@
         <v>1</v>
       </c>
       <c r="D42">
-        <v>1992</v>
+        <v>2004</v>
       </c>
       <c r="E42">
         <v>6</v>
@@ -36868,10 +36868,10 @@
         <v>1</v>
       </c>
       <c r="H42">
-        <v>6643.437096</v>
+        <v>5499.954999</v>
       </c>
       <c r="I42">
-        <v>0.06902181079972704</v>
+        <v>0.06319099382871152</v>
       </c>
     </row>
     <row r="43">
@@ -36887,7 +36887,7 @@
         <v>1</v>
       </c>
       <c r="D43">
-        <v>1993</v>
+        <v>2005</v>
       </c>
       <c r="E43">
         <v>6</v>
@@ -36899,10 +36899,10 @@
         <v>1</v>
       </c>
       <c r="H43">
-        <v>7849.269927</v>
+        <v>6972.381231</v>
       </c>
       <c r="I43">
-        <v>0.06360506917753753</v>
+        <v>0.06657770931057111</v>
       </c>
     </row>
     <row r="44">
@@ -36918,7 +36918,7 @@
         <v>1</v>
       </c>
       <c r="D44">
-        <v>1994</v>
+        <v>2006</v>
       </c>
       <c r="E44">
         <v>6</v>
@@ -36930,10 +36930,10 @@
         <v>1</v>
       </c>
       <c r="H44">
-        <v>7094.434902</v>
+        <v>4190.345627</v>
       </c>
       <c r="I44">
-        <v>0.06544262343842422</v>
+        <v>0.06481560164153972</v>
       </c>
     </row>
     <row r="45">
@@ -36949,7 +36949,7 @@
         <v>1</v>
       </c>
       <c r="D45">
-        <v>1995</v>
+        <v>2007</v>
       </c>
       <c r="E45">
         <v>6</v>
@@ -36961,10 +36961,10 @@
         <v>1</v>
       </c>
       <c r="H45">
-        <v>6597.187752</v>
+        <v>6777.45227</v>
       </c>
       <c r="I45">
-        <v>0.08288083056818238</v>
+        <v>0.08001857686265934</v>
       </c>
     </row>
     <row r="46">
@@ -36980,7 +36980,7 @@
         <v>1</v>
       </c>
       <c r="D46">
-        <v>1996</v>
+        <v>2008</v>
       </c>
       <c r="E46">
         <v>6</v>
@@ -36992,10 +36992,10 @@
         <v>1</v>
       </c>
       <c r="H46">
-        <v>3954.25528</v>
+        <v>4293.26099</v>
       </c>
       <c r="I46">
-        <v>0.06123113690322998</v>
+        <v>0.07804899932254061</v>
       </c>
     </row>
     <row r="47">
@@ -37011,7 +37011,7 @@
         <v>1</v>
       </c>
       <c r="D47">
-        <v>1997</v>
+        <v>2009</v>
       </c>
       <c r="E47">
         <v>6</v>
@@ -37023,10 +37023,10 @@
         <v>1</v>
       </c>
       <c r="H47">
-        <v>4371.517782</v>
+        <v>2820.215503</v>
       </c>
       <c r="I47">
-        <v>0.062961542929851</v>
+        <v>0.08077968572176876</v>
       </c>
     </row>
     <row r="48">
@@ -37042,7 +37042,7 @@
         <v>1</v>
       </c>
       <c r="D48">
-        <v>1998</v>
+        <v>2010</v>
       </c>
       <c r="E48">
         <v>6</v>
@@ -37054,10 +37054,10 @@
         <v>1</v>
       </c>
       <c r="H48">
-        <v>3417.606809</v>
+        <v>5271.619717</v>
       </c>
       <c r="I48">
-        <v>0.06118056598827428</v>
+        <v>0.07818006226263609</v>
       </c>
     </row>
     <row r="49">
@@ -37073,7 +37073,7 @@
         <v>1</v>
       </c>
       <c r="D49">
-        <v>1999</v>
+        <v>2011</v>
       </c>
       <c r="E49">
         <v>6</v>
@@ -37085,10 +37085,10 @@
         <v>1</v>
       </c>
       <c r="H49">
-        <v>5613.644193</v>
+        <v>4505.989345</v>
       </c>
       <c r="I49">
-        <v>0.07159299908981602</v>
+        <v>0.07112668829446599</v>
       </c>
     </row>
     <row r="50">
@@ -37104,7 +37104,7 @@
         <v>1</v>
       </c>
       <c r="D50">
-        <v>2000</v>
+        <v>2012</v>
       </c>
       <c r="E50">
         <v>6</v>
@@ -37116,10 +37116,10 @@
         <v>1</v>
       </c>
       <c r="H50">
-        <v>7246.347745</v>
+        <v>5144.393306</v>
       </c>
       <c r="I50">
-        <v>0.07060087017670444</v>
+        <v>0.0645661033561729</v>
       </c>
     </row>
     <row r="51">
@@ -37135,7 +37135,7 @@
         <v>1</v>
       </c>
       <c r="D51">
-        <v>2001</v>
+        <v>2013</v>
       </c>
       <c r="E51">
         <v>6</v>
@@ -37147,10 +37147,10 @@
         <v>1</v>
       </c>
       <c r="H51">
-        <v>6066.56982</v>
+        <v>6712.589766</v>
       </c>
       <c r="I51">
-        <v>0.06576865219363782</v>
+        <v>0.06473511855304998</v>
       </c>
     </row>
     <row r="52">
@@ -37166,7 +37166,7 @@
         <v>1</v>
       </c>
       <c r="D52">
-        <v>2002</v>
+        <v>2014</v>
       </c>
       <c r="E52">
         <v>6</v>
@@ -37178,10 +37178,10 @@
         <v>1</v>
       </c>
       <c r="H52">
-        <v>6740.603163</v>
+        <v>11616.5106</v>
       </c>
       <c r="I52">
-        <v>0.05824869705358147</v>
+        <v>0.05611087505915933</v>
       </c>
     </row>
     <row r="53">
@@ -37197,7 +37197,7 @@
         <v>1</v>
       </c>
       <c r="D53">
-        <v>2003</v>
+        <v>2015</v>
       </c>
       <c r="E53">
         <v>6</v>
@@ -37209,10 +37209,10 @@
         <v>1</v>
       </c>
       <c r="H53">
-        <v>11239.16293</v>
+        <v>11215.70685</v>
       </c>
       <c r="I53">
-        <v>0.06842173667109566</v>
+        <v>0.05978009315569798</v>
       </c>
     </row>
     <row r="54">
@@ -37228,7 +37228,7 @@
         <v>1</v>
       </c>
       <c r="D54">
-        <v>2004</v>
+        <v>2016</v>
       </c>
       <c r="E54">
         <v>6</v>
@@ -37240,10 +37240,10 @@
         <v>1</v>
       </c>
       <c r="H54">
-        <v>5499.954999</v>
+        <v>8274.5087</v>
       </c>
       <c r="I54">
-        <v>0.06319099382871152</v>
+        <v>0.06958376391579599</v>
       </c>
     </row>
     <row r="55">
@@ -37259,7 +37259,7 @@
         <v>1</v>
       </c>
       <c r="D55">
-        <v>2005</v>
+        <v>2017</v>
       </c>
       <c r="E55">
         <v>6</v>
@@ -37271,10 +37271,10 @@
         <v>1</v>
       </c>
       <c r="H55">
-        <v>6972.381231</v>
+        <v>8855.042158</v>
       </c>
       <c r="I55">
-        <v>0.06657770931057111</v>
+        <v>0.05100407413554405</v>
       </c>
     </row>
     <row r="56">
@@ -37290,7 +37290,7 @@
         <v>1</v>
       </c>
       <c r="D56">
-        <v>2006</v>
+        <v>2018</v>
       </c>
       <c r="E56">
         <v>6</v>
@@ -37302,10 +37302,10 @@
         <v>1</v>
       </c>
       <c r="H56">
-        <v>4190.345627</v>
+        <v>4266.875366</v>
       </c>
       <c r="I56">
-        <v>0.06481560164153972</v>
+        <v>0.06789336686709306</v>
       </c>
     </row>
     <row r="57">
@@ -37321,7 +37321,7 @@
         <v>1</v>
       </c>
       <c r="D57">
-        <v>2007</v>
+        <v>2019</v>
       </c>
       <c r="E57">
         <v>6</v>
@@ -37333,10 +37333,10 @@
         <v>1</v>
       </c>
       <c r="H57">
-        <v>6777.45227</v>
+        <v>9257.419352000001</v>
       </c>
       <c r="I57">
-        <v>0.08001857686265934</v>
+        <v>0.05017169504151895</v>
       </c>
     </row>
     <row r="58">
@@ -37352,7 +37352,7 @@
         <v>1</v>
       </c>
       <c r="D58">
-        <v>2008</v>
+        <v>2021</v>
       </c>
       <c r="E58">
         <v>6</v>
@@ -37364,10 +37364,10 @@
         <v>1</v>
       </c>
       <c r="H58">
-        <v>4293.26099</v>
+        <v>4889.162547</v>
       </c>
       <c r="I58">
-        <v>0.07804899932254061</v>
+        <v>0.05370632877835469</v>
       </c>
     </row>
     <row r="59">
@@ -37383,7 +37383,7 @@
         <v>1</v>
       </c>
       <c r="D59">
-        <v>2009</v>
+        <v>2022</v>
       </c>
       <c r="E59">
         <v>6</v>
@@ -37395,10 +37395,10 @@
         <v>1</v>
       </c>
       <c r="H59">
-        <v>2820.215503</v>
+        <v>6531.432089</v>
       </c>
       <c r="I59">
-        <v>0.08077968572176876</v>
+        <v>0.05876100606578626</v>
       </c>
     </row>
     <row r="60">
@@ -37414,7 +37414,7 @@
         <v>1</v>
       </c>
       <c r="D60">
-        <v>2010</v>
+        <v>2023</v>
       </c>
       <c r="E60">
         <v>6</v>
@@ -37426,10 +37426,10 @@
         <v>1</v>
       </c>
       <c r="H60">
-        <v>5271.619717</v>
+        <v>4945.387531</v>
       </c>
       <c r="I60">
-        <v>0.07818006226263609</v>
+        <v>0.05711794595051321</v>
       </c>
     </row>
     <row r="61">
@@ -37445,7 +37445,7 @@
         <v>1</v>
       </c>
       <c r="D61">
-        <v>2011</v>
+        <v>2024</v>
       </c>
       <c r="E61">
         <v>6</v>
@@ -37457,26 +37457,26 @@
         <v>1</v>
       </c>
       <c r="H61">
-        <v>4505.989345</v>
+        <v>9407.463571</v>
       </c>
       <c r="I61">
-        <v>0.07112668829446599</v>
+        <v>0.07692068051485203</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>BTS</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="B62">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C62">
         <v>1</v>
       </c>
       <c r="D62">
-        <v>2012</v>
+        <v>1994</v>
       </c>
       <c r="E62">
         <v>6</v>
@@ -37488,26 +37488,26 @@
         <v>1</v>
       </c>
       <c r="H62">
-        <v>5144.393306</v>
+        <v>3628.9293</v>
       </c>
       <c r="I62">
-        <v>0.0645661033561729</v>
+        <v>0.1890055559914049</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>BTS</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="B63">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C63">
         <v>1</v>
       </c>
       <c r="D63">
-        <v>2013</v>
+        <v>1996</v>
       </c>
       <c r="E63">
         <v>6</v>
@@ -37519,26 +37519,26 @@
         <v>1</v>
       </c>
       <c r="H63">
-        <v>6712.589766</v>
+        <v>2944.77187</v>
       </c>
       <c r="I63">
-        <v>0.06473511855304998</v>
+        <v>0.1486974201502407</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>BTS</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="B64">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C64">
         <v>1</v>
       </c>
       <c r="D64">
-        <v>2014</v>
+        <v>1997</v>
       </c>
       <c r="E64">
         <v>6</v>
@@ -37550,26 +37550,26 @@
         <v>1</v>
       </c>
       <c r="H64">
-        <v>11616.5106</v>
+        <v>3590.84054</v>
       </c>
       <c r="I64">
-        <v>0.05611087505915933</v>
+        <v>0.1353304260066085</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>BTS</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="B65">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C65">
         <v>1</v>
       </c>
       <c r="D65">
-        <v>2015</v>
+        <v>1999</v>
       </c>
       <c r="E65">
         <v>6</v>
@@ -37581,26 +37581,26 @@
         <v>1</v>
       </c>
       <c r="H65">
-        <v>11215.70685</v>
+        <v>4141.37057</v>
       </c>
       <c r="I65">
-        <v>0.05978009315569798</v>
+        <v>0.2043826592412376</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>BTS</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="B66">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C66">
         <v>1</v>
       </c>
       <c r="D66">
-        <v>2016</v>
+        <v>2000</v>
       </c>
       <c r="E66">
         <v>6</v>
@@ -37612,26 +37612,26 @@
         <v>1</v>
       </c>
       <c r="H66">
-        <v>8274.5087</v>
+        <v>3625.86364</v>
       </c>
       <c r="I66">
-        <v>0.06958376391579599</v>
+        <v>0.128670997125529</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>BTS</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="B67">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C67">
         <v>1</v>
       </c>
       <c r="D67">
-        <v>2017</v>
+        <v>2002</v>
       </c>
       <c r="E67">
         <v>6</v>
@@ -37643,26 +37643,26 @@
         <v>1</v>
       </c>
       <c r="H67">
-        <v>8855.042158</v>
+        <v>4305.86229</v>
       </c>
       <c r="I67">
-        <v>0.05100407413554405</v>
+        <v>0.1244069675066176</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>BTS</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="B68">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C68">
         <v>1</v>
       </c>
       <c r="D68">
-        <v>2018</v>
+        <v>2004</v>
       </c>
       <c r="E68">
         <v>6</v>
@@ -37674,26 +37674,26 @@
         <v>1</v>
       </c>
       <c r="H68">
-        <v>4266.875366</v>
+        <v>4009.93704</v>
       </c>
       <c r="I68">
-        <v>0.06789336686709306</v>
+        <v>0.1444254097316201</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>BTS</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="B69">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C69">
         <v>1</v>
       </c>
       <c r="D69">
-        <v>2019</v>
+        <v>2006</v>
       </c>
       <c r="E69">
         <v>6</v>
@@ -37705,26 +37705,26 @@
         <v>1</v>
       </c>
       <c r="H69">
-        <v>9257.419352000001</v>
+        <v>1872.86327</v>
       </c>
       <c r="I69">
-        <v>0.05017169504151895</v>
+        <v>0.1565715739622573</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>BTS</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="B70">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C70">
         <v>1</v>
       </c>
       <c r="D70">
-        <v>2021</v>
+        <v>2007</v>
       </c>
       <c r="E70">
         <v>6</v>
@@ -37736,26 +37736,26 @@
         <v>1</v>
       </c>
       <c r="H70">
-        <v>4889.162547</v>
+        <v>2277.944</v>
       </c>
       <c r="I70">
-        <v>0.05370632877835469</v>
+        <v>0.1754534571525903</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>BTS</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="B71">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C71">
         <v>1</v>
       </c>
       <c r="D71">
-        <v>2022</v>
+        <v>2008</v>
       </c>
       <c r="E71">
         <v>6</v>
@@ -37767,26 +37767,26 @@
         <v>1</v>
       </c>
       <c r="H71">
-        <v>6531.432089</v>
+        <v>1405.59025</v>
       </c>
       <c r="I71">
-        <v>0.05876100606578626</v>
+        <v>0.2603814945358365</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>BTS</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="B72">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C72">
         <v>1</v>
       </c>
       <c r="D72">
-        <v>2023</v>
+        <v>2009</v>
       </c>
       <c r="E72">
         <v>6</v>
@@ -37798,26 +37798,26 @@
         <v>1</v>
       </c>
       <c r="H72">
-        <v>4945.387531</v>
+        <v>1324.78137</v>
       </c>
       <c r="I72">
-        <v>0.05711794595051321</v>
+        <v>0.3209667116620156</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>BTS</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="B73">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C73">
         <v>1</v>
       </c>
       <c r="D73">
-        <v>2024</v>
+        <v>2010</v>
       </c>
       <c r="E73">
         <v>6</v>
@@ -37829,10 +37829,10 @@
         <v>1</v>
       </c>
       <c r="H73">
-        <v>9407.463571</v>
+        <v>2642.6749</v>
       </c>
       <c r="I73">
-        <v>0.07692068051485203</v>
+        <v>0.250335612602216</v>
       </c>
     </row>
     <row r="74">
@@ -37848,7 +37848,7 @@
         <v>1</v>
       </c>
       <c r="D74">
-        <v>1994</v>
+        <v>2012</v>
       </c>
       <c r="E74">
         <v>6</v>
@@ -37860,10 +37860,10 @@
         <v>1</v>
       </c>
       <c r="H74">
-        <v>3628.9293</v>
+        <v>2295.95185</v>
       </c>
       <c r="I74">
-        <v>0.1890055559914049</v>
+        <v>0.1591845839449987</v>
       </c>
     </row>
     <row r="75">
@@ -37879,7 +37879,7 @@
         <v>1</v>
       </c>
       <c r="D75">
-        <v>1996</v>
+        <v>2014</v>
       </c>
       <c r="E75">
         <v>6</v>
@@ -37891,10 +37891,10 @@
         <v>1</v>
       </c>
       <c r="H75">
-        <v>2944.77187</v>
+        <v>4729.82772</v>
       </c>
       <c r="I75">
-        <v>0.1486974201502407</v>
+        <v>0.1610945778803123</v>
       </c>
     </row>
     <row r="76">
@@ -37910,7 +37910,7 @@
         <v>1</v>
       </c>
       <c r="D76">
-        <v>1997</v>
+        <v>2016</v>
       </c>
       <c r="E76">
         <v>6</v>
@@ -37922,10 +37922,10 @@
         <v>1</v>
       </c>
       <c r="H76">
-        <v>3590.84054</v>
+        <v>4828.79348</v>
       </c>
       <c r="I76">
-        <v>0.1353304260066085</v>
+        <v>0.08740508198333634</v>
       </c>
     </row>
     <row r="77">
@@ -37941,7 +37941,7 @@
         <v>1</v>
       </c>
       <c r="D77">
-        <v>1999</v>
+        <v>2018</v>
       </c>
       <c r="E77">
         <v>6</v>
@@ -37953,10 +37953,10 @@
         <v>1</v>
       </c>
       <c r="H77">
-        <v>4141.37057</v>
+        <v>2499.40106</v>
       </c>
       <c r="I77">
-        <v>0.2043826592412376</v>
+        <v>0.1843558992489185</v>
       </c>
     </row>
     <row r="78">
@@ -37972,7 +37972,7 @@
         <v>1</v>
       </c>
       <c r="D78">
-        <v>2000</v>
+        <v>2020</v>
       </c>
       <c r="E78">
         <v>6</v>
@@ -37984,10 +37984,10 @@
         <v>1</v>
       </c>
       <c r="H78">
-        <v>3625.86364</v>
+        <v>3617</v>
       </c>
       <c r="I78">
-        <v>0.128670997125529</v>
+        <v>0.4493864860381532</v>
       </c>
     </row>
     <row r="79">
@@ -38003,7 +38003,7 @@
         <v>1</v>
       </c>
       <c r="D79">
-        <v>2002</v>
+        <v>2022</v>
       </c>
       <c r="E79">
         <v>6</v>
@@ -38015,10 +38015,10 @@
         <v>1</v>
       </c>
       <c r="H79">
-        <v>4305.86229</v>
+        <v>3834.04251</v>
       </c>
       <c r="I79">
-        <v>0.1244069675066176</v>
+        <v>0.3203175099902583</v>
       </c>
     </row>
     <row r="80">
@@ -38034,7 +38034,7 @@
         <v>1</v>
       </c>
       <c r="D80">
-        <v>2004</v>
+        <v>2024</v>
       </c>
       <c r="E80">
         <v>6</v>
@@ -38046,26 +38046,26 @@
         <v>1</v>
       </c>
       <c r="H80">
-        <v>4009.93704</v>
+        <v>2870.636995</v>
       </c>
       <c r="I80">
-        <v>0.1444254097316201</v>
+        <v>0.2628487802234291</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>BTS_1</t>
         </is>
       </c>
       <c r="B81">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C81">
         <v>1</v>
       </c>
       <c r="D81">
-        <v>2006</v>
+        <v>1982</v>
       </c>
       <c r="E81">
         <v>6</v>
@@ -38077,26 +38077,26 @@
         <v>1</v>
       </c>
       <c r="H81">
-        <v>1872.86327</v>
+        <v>10950974.45</v>
       </c>
       <c r="I81">
-        <v>0.1565715739622573</v>
+        <v>1</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>BTS_1</t>
         </is>
       </c>
       <c r="B82">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C82">
         <v>1</v>
       </c>
       <c r="D82">
-        <v>2007</v>
+        <v>1983</v>
       </c>
       <c r="E82">
         <v>6</v>
@@ -38108,26 +38108,26 @@
         <v>1</v>
       </c>
       <c r="H82">
-        <v>2277.944</v>
+        <v>45353039.8</v>
       </c>
       <c r="I82">
-        <v>0.1754534571525903</v>
+        <v>1</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>BTS_1</t>
         </is>
       </c>
       <c r="B83">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C83">
         <v>1</v>
       </c>
       <c r="D83">
-        <v>2008</v>
+        <v>1984</v>
       </c>
       <c r="E83">
         <v>6</v>
@@ -38139,26 +38139,26 @@
         <v>1</v>
       </c>
       <c r="H83">
-        <v>1405.59025</v>
+        <v>4810111.378</v>
       </c>
       <c r="I83">
-        <v>0.2603814945358365</v>
+        <v>1</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>BTS_1</t>
         </is>
       </c>
       <c r="B84">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C84">
         <v>1</v>
       </c>
       <c r="D84">
-        <v>2009</v>
+        <v>1985</v>
       </c>
       <c r="E84">
         <v>6</v>
@@ -38170,26 +38170,26 @@
         <v>1</v>
       </c>
       <c r="H84">
-        <v>1324.78137</v>
+        <v>49329672.64</v>
       </c>
       <c r="I84">
-        <v>0.3209667116620156</v>
+        <v>1</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>BTS_1</t>
         </is>
       </c>
       <c r="B85">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C85">
         <v>1</v>
       </c>
       <c r="D85">
-        <v>2010</v>
+        <v>1986</v>
       </c>
       <c r="E85">
         <v>6</v>
@@ -38201,26 +38201,26 @@
         <v>1</v>
       </c>
       <c r="H85">
-        <v>2642.6749</v>
+        <v>29490315.26</v>
       </c>
       <c r="I85">
-        <v>0.250335612602216</v>
+        <v>1</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>BTS_1</t>
         </is>
       </c>
       <c r="B86">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C86">
         <v>1</v>
       </c>
       <c r="D86">
-        <v>2012</v>
+        <v>1987</v>
       </c>
       <c r="E86">
         <v>6</v>
@@ -38232,26 +38232,26 @@
         <v>1</v>
       </c>
       <c r="H86">
-        <v>2295.95185</v>
+        <v>4901555.37</v>
       </c>
       <c r="I86">
-        <v>0.1591845839449987</v>
+        <v>1</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>BTS_1</t>
         </is>
       </c>
       <c r="B87">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C87">
         <v>1</v>
       </c>
       <c r="D87">
-        <v>2014</v>
+        <v>1988</v>
       </c>
       <c r="E87">
         <v>6</v>
@@ -38263,26 +38263,26 @@
         <v>1</v>
       </c>
       <c r="H87">
-        <v>4729.82772</v>
+        <v>15721198.77</v>
       </c>
       <c r="I87">
-        <v>0.1610945778803123</v>
+        <v>1</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>BTS_1</t>
         </is>
       </c>
       <c r="B88">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C88">
         <v>1</v>
       </c>
       <c r="D88">
-        <v>2016</v>
+        <v>1989</v>
       </c>
       <c r="E88">
         <v>6</v>
@@ -38294,26 +38294,26 @@
         <v>1</v>
       </c>
       <c r="H88">
-        <v>4828.79348</v>
+        <v>9045388.605</v>
       </c>
       <c r="I88">
-        <v>0.08740508198333634</v>
+        <v>1</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>BTS_1</t>
         </is>
       </c>
       <c r="B89">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C89">
         <v>1</v>
       </c>
       <c r="D89">
-        <v>2018</v>
+        <v>1990</v>
       </c>
       <c r="E89">
         <v>6</v>
@@ -38325,26 +38325,26 @@
         <v>1</v>
       </c>
       <c r="H89">
-        <v>2499.40106</v>
+        <v>22226901.34</v>
       </c>
       <c r="I89">
-        <v>0.1843558992489185</v>
+        <v>1</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>BTS_1</t>
         </is>
       </c>
       <c r="B90">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C90">
         <v>1</v>
       </c>
       <c r="D90">
-        <v>2020</v>
+        <v>1991</v>
       </c>
       <c r="E90">
         <v>6</v>
@@ -38356,26 +38356,26 @@
         <v>1</v>
       </c>
       <c r="H90">
-        <v>3617</v>
+        <v>32298906.47</v>
       </c>
       <c r="I90">
-        <v>0.4493864860381532</v>
+        <v>1</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>BTS_1</t>
         </is>
       </c>
       <c r="B91">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C91">
         <v>1</v>
       </c>
       <c r="D91">
-        <v>2022</v>
+        <v>1992</v>
       </c>
       <c r="E91">
         <v>6</v>
@@ -38387,26 +38387,26 @@
         <v>1</v>
       </c>
       <c r="H91">
-        <v>3834.04251</v>
+        <v>15591259.43</v>
       </c>
       <c r="I91">
-        <v>0.3203175099902583</v>
+        <v>1</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>BTS_1</t>
         </is>
       </c>
       <c r="B92">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C92">
         <v>1</v>
       </c>
       <c r="D92">
-        <v>2024</v>
+        <v>1993</v>
       </c>
       <c r="E92">
         <v>6</v>
@@ -38418,10 +38418,10 @@
         <v>1</v>
       </c>
       <c r="H92">
-        <v>2870.636995</v>
+        <v>26831974.61</v>
       </c>
       <c r="I92">
-        <v>0.2628487802234291</v>
+        <v>1</v>
       </c>
     </row>
     <row r="93">
@@ -38437,7 +38437,7 @@
         <v>1</v>
       </c>
       <c r="D93">
-        <v>1982</v>
+        <v>1994</v>
       </c>
       <c r="E93">
         <v>6</v>
@@ -38449,7 +38449,7 @@
         <v>1</v>
       </c>
       <c r="H93">
-        <v>10950974.45</v>
+        <v>16300489.78</v>
       </c>
       <c r="I93">
         <v>1</v>
@@ -38468,7 +38468,7 @@
         <v>1</v>
       </c>
       <c r="D94">
-        <v>1983</v>
+        <v>1995</v>
       </c>
       <c r="E94">
         <v>6</v>
@@ -38480,7 +38480,7 @@
         <v>1</v>
       </c>
       <c r="H94">
-        <v>45353039.8</v>
+        <v>16172066.37</v>
       </c>
       <c r="I94">
         <v>1</v>
@@ -38499,7 +38499,7 @@
         <v>1</v>
       </c>
       <c r="D95">
-        <v>1984</v>
+        <v>1996</v>
       </c>
       <c r="E95">
         <v>6</v>
@@ -38511,7 +38511,7 @@
         <v>1</v>
       </c>
       <c r="H95">
-        <v>4810111.378</v>
+        <v>19509804.11</v>
       </c>
       <c r="I95">
         <v>1</v>
@@ -38530,7 +38530,7 @@
         <v>1</v>
       </c>
       <c r="D96">
-        <v>1985</v>
+        <v>1997</v>
       </c>
       <c r="E96">
         <v>6</v>
@@ -38542,7 +38542,7 @@
         <v>1</v>
       </c>
       <c r="H96">
-        <v>49329672.64</v>
+        <v>23321877.34</v>
       </c>
       <c r="I96">
         <v>1</v>
@@ -38561,7 +38561,7 @@
         <v>1</v>
       </c>
       <c r="D97">
-        <v>1986</v>
+        <v>1998</v>
       </c>
       <c r="E97">
         <v>6</v>
@@ -38573,7 +38573,7 @@
         <v>1</v>
       </c>
       <c r="H97">
-        <v>29490315.26</v>
+        <v>8710506.469000001</v>
       </c>
       <c r="I97">
         <v>1</v>
@@ -38592,7 +38592,7 @@
         <v>1</v>
       </c>
       <c r="D98">
-        <v>1987</v>
+        <v>1999</v>
       </c>
       <c r="E98">
         <v>6</v>
@@ -38604,7 +38604,7 @@
         <v>1</v>
       </c>
       <c r="H98">
-        <v>4901555.37</v>
+        <v>9913042.828</v>
       </c>
       <c r="I98">
         <v>1</v>
@@ -38623,7 +38623,7 @@
         <v>1</v>
       </c>
       <c r="D99">
-        <v>1988</v>
+        <v>2000</v>
       </c>
       <c r="E99">
         <v>6</v>
@@ -38635,7 +38635,7 @@
         <v>1</v>
       </c>
       <c r="H99">
-        <v>15721198.77</v>
+        <v>10448664.91</v>
       </c>
       <c r="I99">
         <v>1</v>
@@ -38654,7 +38654,7 @@
         <v>1</v>
       </c>
       <c r="D100">
-        <v>1989</v>
+        <v>2001</v>
       </c>
       <c r="E100">
         <v>6</v>
@@ -38666,7 +38666,7 @@
         <v>1</v>
       </c>
       <c r="H100">
-        <v>9045388.605</v>
+        <v>19866054.3</v>
       </c>
       <c r="I100">
         <v>1</v>
@@ -38685,7 +38685,7 @@
         <v>1</v>
       </c>
       <c r="D101">
-        <v>1990</v>
+        <v>2002</v>
       </c>
       <c r="E101">
         <v>6</v>
@@ -38697,7 +38697,7 @@
         <v>1</v>
       </c>
       <c r="H101">
-        <v>22226901.34</v>
+        <v>13635855.02</v>
       </c>
       <c r="I101">
         <v>1</v>
@@ -38716,7 +38716,7 @@
         <v>1</v>
       </c>
       <c r="D102">
-        <v>1991</v>
+        <v>2003</v>
       </c>
       <c r="E102">
         <v>6</v>
@@ -38728,7 +38728,7 @@
         <v>1</v>
       </c>
       <c r="H102">
-        <v>32298906.47</v>
+        <v>5737576.96</v>
       </c>
       <c r="I102">
         <v>1</v>
@@ -38747,7 +38747,7 @@
         <v>1</v>
       </c>
       <c r="D103">
-        <v>1992</v>
+        <v>2004</v>
       </c>
       <c r="E103">
         <v>6</v>
@@ -38759,7 +38759,7 @@
         <v>1</v>
       </c>
       <c r="H103">
-        <v>15591259.43</v>
+        <v>3971309.628</v>
       </c>
       <c r="I103">
         <v>1</v>
@@ -38778,7 +38778,7 @@
         <v>1</v>
       </c>
       <c r="D104">
-        <v>1993</v>
+        <v>2005</v>
       </c>
       <c r="E104">
         <v>6</v>
@@ -38790,7 +38790,7 @@
         <v>1</v>
       </c>
       <c r="H104">
-        <v>26831974.61</v>
+        <v>4008208.162</v>
       </c>
       <c r="I104">
         <v>1</v>
@@ -38809,7 +38809,7 @@
         <v>1</v>
       </c>
       <c r="D105">
-        <v>1994</v>
+        <v>2006</v>
       </c>
       <c r="E105">
         <v>6</v>
@@ -38821,7 +38821,7 @@
         <v>1</v>
       </c>
       <c r="H105">
-        <v>16300489.78</v>
+        <v>8156013.515</v>
       </c>
       <c r="I105">
         <v>1</v>
@@ -38840,7 +38840,7 @@
         <v>1</v>
       </c>
       <c r="D106">
-        <v>1995</v>
+        <v>2007</v>
       </c>
       <c r="E106">
         <v>6</v>
@@ -38852,7 +38852,7 @@
         <v>1</v>
       </c>
       <c r="H106">
-        <v>16172066.37</v>
+        <v>27341965.7</v>
       </c>
       <c r="I106">
         <v>1</v>
@@ -38871,7 +38871,7 @@
         <v>1</v>
       </c>
       <c r="D107">
-        <v>1996</v>
+        <v>2008</v>
       </c>
       <c r="E107">
         <v>6</v>
@@ -38883,7 +38883,7 @@
         <v>1</v>
       </c>
       <c r="H107">
-        <v>19509804.11</v>
+        <v>5026908.871</v>
       </c>
       <c r="I107">
         <v>1</v>
@@ -38902,7 +38902,7 @@
         <v>1</v>
       </c>
       <c r="D108">
-        <v>1997</v>
+        <v>2009</v>
       </c>
       <c r="E108">
         <v>6</v>
@@ -38914,7 +38914,7 @@
         <v>1</v>
       </c>
       <c r="H108">
-        <v>23321877.34</v>
+        <v>8423248.112</v>
       </c>
       <c r="I108">
         <v>1</v>
@@ -38933,7 +38933,7 @@
         <v>1</v>
       </c>
       <c r="D109">
-        <v>1998</v>
+        <v>2010</v>
       </c>
       <c r="E109">
         <v>6</v>
@@ -38945,7 +38945,7 @@
         <v>1</v>
       </c>
       <c r="H109">
-        <v>8710506.469000001</v>
+        <v>4800589.205</v>
       </c>
       <c r="I109">
         <v>1</v>
@@ -38964,7 +38964,7 @@
         <v>1</v>
       </c>
       <c r="D110">
-        <v>1999</v>
+        <v>2011</v>
       </c>
       <c r="E110">
         <v>6</v>
@@ -38976,7 +38976,7 @@
         <v>1</v>
       </c>
       <c r="H110">
-        <v>9913042.828</v>
+        <v>12920051.51</v>
       </c>
       <c r="I110">
         <v>1</v>
@@ -38995,7 +38995,7 @@
         <v>1</v>
       </c>
       <c r="D111">
-        <v>2000</v>
+        <v>2012</v>
       </c>
       <c r="E111">
         <v>6</v>
@@ -39007,7 +39007,7 @@
         <v>1</v>
       </c>
       <c r="H111">
-        <v>10448664.91</v>
+        <v>12972591.79</v>
       </c>
       <c r="I111">
         <v>1</v>
@@ -39026,7 +39026,7 @@
         <v>1</v>
       </c>
       <c r="D112">
-        <v>2001</v>
+        <v>2013</v>
       </c>
       <c r="E112">
         <v>6</v>
@@ -39038,7 +39038,7 @@
         <v>1</v>
       </c>
       <c r="H112">
-        <v>19866054.3</v>
+        <v>12516351.14</v>
       </c>
       <c r="I112">
         <v>1</v>
@@ -39057,7 +39057,7 @@
         <v>1</v>
       </c>
       <c r="D113">
-        <v>2002</v>
+        <v>2014</v>
       </c>
       <c r="E113">
         <v>6</v>
@@ -39069,7 +39069,7 @@
         <v>1</v>
       </c>
       <c r="H113">
-        <v>13635855.02</v>
+        <v>25378686.14</v>
       </c>
       <c r="I113">
         <v>1</v>
@@ -39088,7 +39088,7 @@
         <v>1</v>
       </c>
       <c r="D114">
-        <v>2003</v>
+        <v>2015</v>
       </c>
       <c r="E114">
         <v>6</v>
@@ -39100,7 +39100,7 @@
         <v>1</v>
       </c>
       <c r="H114">
-        <v>5737576.96</v>
+        <v>14570602.84</v>
       </c>
       <c r="I114">
         <v>1</v>
@@ -39119,7 +39119,7 @@
         <v>1</v>
       </c>
       <c r="D115">
-        <v>2004</v>
+        <v>2016</v>
       </c>
       <c r="E115">
         <v>6</v>
@@ -39131,7 +39131,7 @@
         <v>1</v>
       </c>
       <c r="H115">
-        <v>3971309.628</v>
+        <v>7941441.528</v>
       </c>
       <c r="I115">
         <v>1</v>
@@ -39150,7 +39150,7 @@
         <v>1</v>
       </c>
       <c r="D116">
-        <v>2005</v>
+        <v>2017</v>
       </c>
       <c r="E116">
         <v>6</v>
@@ -39162,7 +39162,7 @@
         <v>1</v>
       </c>
       <c r="H116">
-        <v>4008208.162</v>
+        <v>7835995.184</v>
       </c>
       <c r="I116">
         <v>1</v>
@@ -39181,7 +39181,7 @@
         <v>1</v>
       </c>
       <c r="D117">
-        <v>2006</v>
+        <v>2018</v>
       </c>
       <c r="E117">
         <v>6</v>
@@ -39193,7 +39193,7 @@
         <v>1</v>
       </c>
       <c r="H117">
-        <v>8156013.515</v>
+        <v>11286192.27</v>
       </c>
       <c r="I117">
         <v>1</v>
@@ -39212,7 +39212,7 @@
         <v>1</v>
       </c>
       <c r="D118">
-        <v>2007</v>
+        <v>2019</v>
       </c>
       <c r="E118">
         <v>6</v>
@@ -39224,7 +39224,7 @@
         <v>1</v>
       </c>
       <c r="H118">
-        <v>27341965.7</v>
+        <v>26795702.01</v>
       </c>
       <c r="I118">
         <v>1</v>
@@ -39243,7 +39243,7 @@
         <v>1</v>
       </c>
       <c r="D119">
-        <v>2008</v>
+        <v>2021</v>
       </c>
       <c r="E119">
         <v>6</v>
@@ -39255,7 +39255,7 @@
         <v>1</v>
       </c>
       <c r="H119">
-        <v>5026908.871</v>
+        <v>10321941.11</v>
       </c>
       <c r="I119">
         <v>1</v>
@@ -39274,7 +39274,7 @@
         <v>1</v>
       </c>
       <c r="D120">
-        <v>2009</v>
+        <v>2022</v>
       </c>
       <c r="E120">
         <v>6</v>
@@ -39286,7 +39286,7 @@
         <v>1</v>
       </c>
       <c r="H120">
-        <v>8423248.112</v>
+        <v>8119155.479</v>
       </c>
       <c r="I120">
         <v>1</v>
@@ -39305,7 +39305,7 @@
         <v>1</v>
       </c>
       <c r="D121">
-        <v>2010</v>
+        <v>2023</v>
       </c>
       <c r="E121">
         <v>6</v>
@@ -39317,7 +39317,7 @@
         <v>1</v>
       </c>
       <c r="H121">
-        <v>4800589.205</v>
+        <v>11137835.36</v>
       </c>
       <c r="I121">
         <v>1</v>
@@ -39336,7 +39336,7 @@
         <v>1</v>
       </c>
       <c r="D122">
-        <v>2011</v>
+        <v>2024</v>
       </c>
       <c r="E122">
         <v>6</v>
@@ -39348,7 +39348,7 @@
         <v>1</v>
       </c>
       <c r="H122">
-        <v>12920051.51</v>
+        <v>16262095.59</v>
       </c>
       <c r="I122">
         <v>1</v>
@@ -39357,17 +39357,17 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>BTS_1</t>
+          <t>ATS_1</t>
         </is>
       </c>
       <c r="B123">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C123">
         <v>1</v>
       </c>
       <c r="D123">
-        <v>2012</v>
+        <v>1994</v>
       </c>
       <c r="E123">
         <v>6</v>
@@ -39379,7 +39379,7 @@
         <v>1</v>
       </c>
       <c r="H123">
-        <v>12972591.79</v>
+        <v>1140.08514</v>
       </c>
       <c r="I123">
         <v>1</v>
@@ -39388,17 +39388,17 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>BTS_1</t>
+          <t>ATS_1</t>
         </is>
       </c>
       <c r="B124">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C124">
         <v>1</v>
       </c>
       <c r="D124">
-        <v>2013</v>
+        <v>1996</v>
       </c>
       <c r="E124">
         <v>6</v>
@@ -39410,7 +39410,7 @@
         <v>1</v>
       </c>
       <c r="H124">
-        <v>12516351.14</v>
+        <v>1800.254055</v>
       </c>
       <c r="I124">
         <v>1</v>
@@ -39419,17 +39419,17 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>BTS_1</t>
+          <t>ATS_1</t>
         </is>
       </c>
       <c r="B125">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C125">
         <v>1</v>
       </c>
       <c r="D125">
-        <v>2014</v>
+        <v>1997</v>
       </c>
       <c r="E125">
         <v>6</v>
@@ -39441,7 +39441,7 @@
         <v>1</v>
       </c>
       <c r="H125">
-        <v>25378686.14</v>
+        <v>13226.7894</v>
       </c>
       <c r="I125">
         <v>1</v>
@@ -39450,17 +39450,17 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>BTS_1</t>
+          <t>ATS_1</t>
         </is>
       </c>
       <c r="B126">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C126">
         <v>1</v>
       </c>
       <c r="D126">
-        <v>2015</v>
+        <v>1999</v>
       </c>
       <c r="E126">
         <v>6</v>
@@ -39472,7 +39472,7 @@
         <v>1</v>
       </c>
       <c r="H126">
-        <v>14570602.84</v>
+        <v>607.203652</v>
       </c>
       <c r="I126">
         <v>1</v>
@@ -39481,17 +39481,17 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>BTS_1</t>
+          <t>ATS_1</t>
         </is>
       </c>
       <c r="B127">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C127">
         <v>1</v>
       </c>
       <c r="D127">
-        <v>2016</v>
+        <v>2000</v>
       </c>
       <c r="E127">
         <v>6</v>
@@ -39503,7 +39503,7 @@
         <v>1</v>
       </c>
       <c r="H127">
-        <v>7941441.528</v>
+        <v>460.3664031</v>
       </c>
       <c r="I127">
         <v>1</v>
@@ -39512,17 +39512,17 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>BTS_1</t>
+          <t>ATS_1</t>
         </is>
       </c>
       <c r="B128">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C128">
         <v>1</v>
       </c>
       <c r="D128">
-        <v>2017</v>
+        <v>2002</v>
       </c>
       <c r="E128">
         <v>6</v>
@@ -39534,7 +39534,7 @@
         <v>1</v>
       </c>
       <c r="H128">
-        <v>7835995.184</v>
+        <v>796.3968503</v>
       </c>
       <c r="I128">
         <v>1</v>
@@ -39543,17 +39543,17 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>BTS_1</t>
+          <t>ATS_1</t>
         </is>
       </c>
       <c r="B129">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C129">
         <v>1</v>
       </c>
       <c r="D129">
-        <v>2018</v>
+        <v>2004</v>
       </c>
       <c r="E129">
         <v>6</v>
@@ -39565,7 +39565,7 @@
         <v>1</v>
       </c>
       <c r="H129">
-        <v>11286192.27</v>
+        <v>83.05449742</v>
       </c>
       <c r="I129">
         <v>1</v>
@@ -39574,17 +39574,17 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>BTS_1</t>
+          <t>ATS_1</t>
         </is>
       </c>
       <c r="B130">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C130">
         <v>1</v>
       </c>
       <c r="D130">
-        <v>2019</v>
+        <v>2006</v>
       </c>
       <c r="E130">
         <v>6</v>
@@ -39596,7 +39596,7 @@
         <v>1</v>
       </c>
       <c r="H130">
-        <v>26795702.01</v>
+        <v>524.7109597</v>
       </c>
       <c r="I130">
         <v>1</v>
@@ -39605,17 +39605,17 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>BTS_1</t>
+          <t>ATS_1</t>
         </is>
       </c>
       <c r="B131">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C131">
         <v>1</v>
       </c>
       <c r="D131">
-        <v>2021</v>
+        <v>2007</v>
       </c>
       <c r="E131">
         <v>6</v>
@@ -39627,7 +39627,7 @@
         <v>1</v>
       </c>
       <c r="H131">
-        <v>10321941.11</v>
+        <v>5775.294145</v>
       </c>
       <c r="I131">
         <v>1</v>
@@ -39636,17 +39636,17 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>BTS_1</t>
+          <t>ATS_1</t>
         </is>
       </c>
       <c r="B132">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C132">
         <v>1</v>
       </c>
       <c r="D132">
-        <v>2022</v>
+        <v>2008</v>
       </c>
       <c r="E132">
         <v>6</v>
@@ -39658,7 +39658,7 @@
         <v>1</v>
       </c>
       <c r="H132">
-        <v>8119155.479</v>
+        <v>70.86987403000001</v>
       </c>
       <c r="I132">
         <v>1</v>
@@ -39667,17 +39667,17 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>BTS_1</t>
+          <t>ATS_1</t>
         </is>
       </c>
       <c r="B133">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C133">
         <v>1</v>
       </c>
       <c r="D133">
-        <v>2023</v>
+        <v>2009</v>
       </c>
       <c r="E133">
         <v>6</v>
@@ -39689,7 +39689,7 @@
         <v>1</v>
       </c>
       <c r="H133">
-        <v>11137835.36</v>
+        <v>5196.786272</v>
       </c>
       <c r="I133">
         <v>1</v>
@@ -39698,17 +39698,17 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>BTS_1</t>
+          <t>ATS_1</t>
         </is>
       </c>
       <c r="B134">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C134">
         <v>1</v>
       </c>
       <c r="D134">
-        <v>2024</v>
+        <v>2010</v>
       </c>
       <c r="E134">
         <v>6</v>
@@ -39720,7 +39720,7 @@
         <v>1</v>
       </c>
       <c r="H134">
-        <v>16262095.59</v>
+        <v>2567.932041</v>
       </c>
       <c r="I134">
         <v>1</v>
@@ -39739,7 +39739,7 @@
         <v>1</v>
       </c>
       <c r="D135">
-        <v>1994</v>
+        <v>2012</v>
       </c>
       <c r="E135">
         <v>6</v>
@@ -39751,7 +39751,7 @@
         <v>1</v>
       </c>
       <c r="H135">
-        <v>1140.08514</v>
+        <v>177.3461428</v>
       </c>
       <c r="I135">
         <v>1</v>
@@ -39770,7 +39770,7 @@
         <v>1</v>
       </c>
       <c r="D136">
-        <v>1996</v>
+        <v>2014</v>
       </c>
       <c r="E136">
         <v>6</v>
@@ -39782,7 +39782,7 @@
         <v>1</v>
       </c>
       <c r="H136">
-        <v>1800.254055</v>
+        <v>4750.826376</v>
       </c>
       <c r="I136">
         <v>1</v>
@@ -39801,7 +39801,7 @@
         <v>1</v>
       </c>
       <c r="D137">
-        <v>1997</v>
+        <v>2016</v>
       </c>
       <c r="E137">
         <v>6</v>
@@ -39813,7 +39813,7 @@
         <v>1</v>
       </c>
       <c r="H137">
-        <v>13226.7894</v>
+        <v>173.7523144</v>
       </c>
       <c r="I137">
         <v>1</v>
@@ -39832,7 +39832,7 @@
         <v>1</v>
       </c>
       <c r="D138">
-        <v>1999</v>
+        <v>2018</v>
       </c>
       <c r="E138">
         <v>6</v>
@@ -39844,7 +39844,7 @@
         <v>1</v>
       </c>
       <c r="H138">
-        <v>607.203652</v>
+        <v>449.9560697</v>
       </c>
       <c r="I138">
         <v>1</v>
@@ -39863,7 +39863,7 @@
         <v>1</v>
       </c>
       <c r="D139">
-        <v>2000</v>
+        <v>2020</v>
       </c>
       <c r="E139">
         <v>6</v>
@@ -39875,7 +39875,7 @@
         <v>1</v>
       </c>
       <c r="H139">
-        <v>460.3664031</v>
+        <v>350</v>
       </c>
       <c r="I139">
         <v>1</v>
@@ -39894,7 +39894,7 @@
         <v>1</v>
       </c>
       <c r="D140">
-        <v>2002</v>
+        <v>2022</v>
       </c>
       <c r="E140">
         <v>6</v>
@@ -39906,7 +39906,7 @@
         <v>1</v>
       </c>
       <c r="H140">
-        <v>796.3968503</v>
+        <v>141.5599371</v>
       </c>
       <c r="I140">
         <v>1</v>
@@ -39925,7 +39925,7 @@
         <v>1</v>
       </c>
       <c r="D141">
-        <v>2004</v>
+        <v>-2024</v>
       </c>
       <c r="E141">
         <v>6</v>
@@ -39937,7 +39937,7 @@
         <v>1</v>
       </c>
       <c r="H141">
-        <v>83.05449742</v>
+        <v>5074.817226</v>
       </c>
       <c r="I141">
         <v>1</v>
@@ -39946,20 +39946,20 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>ATS_1</t>
+          <t>CPUE</t>
         </is>
       </c>
       <c r="B142">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C142">
         <v>1</v>
       </c>
       <c r="D142">
-        <v>2006</v>
+        <v>1965</v>
       </c>
       <c r="E142">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F142">
         <v>1</v>
@@ -39968,29 +39968,29 @@
         <v>1</v>
       </c>
       <c r="H142">
-        <v>524.7109597</v>
+        <v>2816.437428</v>
       </c>
       <c r="I142">
-        <v>1</v>
+        <v>563.2874856</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>ATS_1</t>
+          <t>CPUE</t>
         </is>
       </c>
       <c r="B143">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C143">
         <v>1</v>
       </c>
       <c r="D143">
-        <v>2007</v>
+        <v>1966</v>
       </c>
       <c r="E143">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F143">
         <v>1</v>
@@ -39999,29 +39999,29 @@
         <v>1</v>
       </c>
       <c r="H143">
-        <v>5775.294145</v>
+        <v>3473.580475</v>
       </c>
       <c r="I143">
-        <v>1</v>
+        <v>694.716095</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>ATS_1</t>
+          <t>CPUE</t>
         </is>
       </c>
       <c r="B144">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C144">
         <v>1</v>
       </c>
       <c r="D144">
-        <v>2008</v>
+        <v>1967</v>
       </c>
       <c r="E144">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F144">
         <v>1</v>
@@ -40030,29 +40030,29 @@
         <v>1</v>
       </c>
       <c r="H144">
-        <v>70.86987403000001</v>
+        <v>3802.169891</v>
       </c>
       <c r="I144">
-        <v>1</v>
+        <v>760.4339781</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>ATS_1</t>
+          <t>CPUE</t>
         </is>
       </c>
       <c r="B145">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C145">
         <v>1</v>
       </c>
       <c r="D145">
-        <v>2009</v>
+        <v>1968</v>
       </c>
       <c r="E145">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F145">
         <v>1</v>
@@ -40061,29 +40061,29 @@
         <v>1</v>
       </c>
       <c r="H145">
-        <v>5196.786272</v>
+        <v>5257.304601</v>
       </c>
       <c r="I145">
-        <v>1</v>
+        <v>1051.46092</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>ATS_1</t>
+          <t>CPUE</t>
         </is>
       </c>
       <c r="B146">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C146">
         <v>1</v>
       </c>
       <c r="D146">
-        <v>2010</v>
+        <v>1969</v>
       </c>
       <c r="E146">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F146">
         <v>1</v>
@@ -40092,29 +40092,29 @@
         <v>1</v>
       </c>
       <c r="H146">
-        <v>2567.932041</v>
+        <v>6712.468418</v>
       </c>
       <c r="I146">
-        <v>1</v>
+        <v>1342.493684</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>ATS_1</t>
+          <t>CPUE</t>
         </is>
       </c>
       <c r="B147">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C147">
         <v>1</v>
       </c>
       <c r="D147">
-        <v>2012</v>
+        <v>1970</v>
       </c>
       <c r="E147">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F147">
         <v>1</v>
@@ -40123,29 +40123,29 @@
         <v>1</v>
       </c>
       <c r="H147">
-        <v>177.3461428</v>
+        <v>5679.809828</v>
       </c>
       <c r="I147">
-        <v>1</v>
+        <v>1135.961966</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>ATS_1</t>
+          <t>CPUE</t>
         </is>
       </c>
       <c r="B148">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C148">
         <v>1</v>
       </c>
       <c r="D148">
-        <v>2014</v>
+        <v>1971</v>
       </c>
       <c r="E148">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F148">
         <v>1</v>
@@ -40154,29 +40154,29 @@
         <v>1</v>
       </c>
       <c r="H148">
-        <v>4750.826376</v>
+        <v>5257.331283</v>
       </c>
       <c r="I148">
-        <v>1</v>
+        <v>1051.466257</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>ATS_1</t>
+          <t>CPUE</t>
         </is>
       </c>
       <c r="B149">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C149">
         <v>1</v>
       </c>
       <c r="D149">
-        <v>2016</v>
+        <v>1972</v>
       </c>
       <c r="E149">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F149">
         <v>1</v>
@@ -40185,29 +40185,29 @@
         <v>1</v>
       </c>
       <c r="H149">
-        <v>173.7523144</v>
+        <v>5726.743484</v>
       </c>
       <c r="I149">
-        <v>1</v>
+        <v>1145.348697</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>ATS_1</t>
+          <t>CPUE</t>
         </is>
       </c>
       <c r="B150">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C150">
         <v>1</v>
       </c>
       <c r="D150">
-        <v>2018</v>
+        <v>1973</v>
       </c>
       <c r="E150">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F150">
         <v>1</v>
@@ -40216,29 +40216,29 @@
         <v>1</v>
       </c>
       <c r="H150">
-        <v>449.9560697</v>
+        <v>4787.923949</v>
       </c>
       <c r="I150">
-        <v>1</v>
+        <v>957.5847898</v>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>ATS_1</t>
+          <t>CPUE</t>
         </is>
       </c>
       <c r="B151">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C151">
         <v>1</v>
       </c>
       <c r="D151">
-        <v>2020</v>
+        <v>1974</v>
       </c>
       <c r="E151">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F151">
         <v>1</v>
@@ -40247,29 +40247,29 @@
         <v>1</v>
       </c>
       <c r="H151">
-        <v>350</v>
+        <v>4740.992588</v>
       </c>
       <c r="I151">
-        <v>1</v>
+        <v>948.1985175999999</v>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>ATS_1</t>
+          <t>CPUE</t>
         </is>
       </c>
       <c r="B152">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C152">
         <v>1</v>
       </c>
       <c r="D152">
-        <v>2022</v>
+        <v>1975</v>
       </c>
       <c r="E152">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F152">
         <v>1</v>
@@ -40278,29 +40278,29 @@
         <v>1</v>
       </c>
       <c r="H152">
-        <v>141.5599371</v>
+        <v>4271.57446</v>
       </c>
       <c r="I152">
-        <v>1</v>
+        <v>854.3148919</v>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>ATS_1</t>
+          <t>CPUE</t>
         </is>
       </c>
       <c r="B153">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C153">
         <v>1</v>
       </c>
       <c r="D153">
-        <v>-2024</v>
+        <v>1976</v>
       </c>
       <c r="E153">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F153">
         <v>1</v>
@@ -40309,381 +40309,9 @@
         <v>1</v>
       </c>
       <c r="H153">
-        <v>5074.817226</v>
+        <v>4318.523058</v>
       </c>
       <c r="I153">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="154">
-      <c r="A154" t="inlineStr">
-        <is>
-          <t>CPUE</t>
-        </is>
-      </c>
-      <c r="B154">
-        <v>7</v>
-      </c>
-      <c r="C154">
-        <v>1</v>
-      </c>
-      <c r="D154">
-        <v>1965</v>
-      </c>
-      <c r="E154">
-        <v>0</v>
-      </c>
-      <c r="F154">
-        <v>1</v>
-      </c>
-      <c r="G154">
-        <v>1</v>
-      </c>
-      <c r="H154">
-        <v>2816.437428</v>
-      </c>
-      <c r="I154">
-        <v>563.2874856</v>
-      </c>
-    </row>
-    <row r="155">
-      <c r="A155" t="inlineStr">
-        <is>
-          <t>CPUE</t>
-        </is>
-      </c>
-      <c r="B155">
-        <v>7</v>
-      </c>
-      <c r="C155">
-        <v>1</v>
-      </c>
-      <c r="D155">
-        <v>1966</v>
-      </c>
-      <c r="E155">
-        <v>0</v>
-      </c>
-      <c r="F155">
-        <v>1</v>
-      </c>
-      <c r="G155">
-        <v>1</v>
-      </c>
-      <c r="H155">
-        <v>3473.580475</v>
-      </c>
-      <c r="I155">
-        <v>694.716095</v>
-      </c>
-    </row>
-    <row r="156">
-      <c r="A156" t="inlineStr">
-        <is>
-          <t>CPUE</t>
-        </is>
-      </c>
-      <c r="B156">
-        <v>7</v>
-      </c>
-      <c r="C156">
-        <v>1</v>
-      </c>
-      <c r="D156">
-        <v>1967</v>
-      </c>
-      <c r="E156">
-        <v>0</v>
-      </c>
-      <c r="F156">
-        <v>1</v>
-      </c>
-      <c r="G156">
-        <v>1</v>
-      </c>
-      <c r="H156">
-        <v>3802.169891</v>
-      </c>
-      <c r="I156">
-        <v>760.4339781</v>
-      </c>
-    </row>
-    <row r="157">
-      <c r="A157" t="inlineStr">
-        <is>
-          <t>CPUE</t>
-        </is>
-      </c>
-      <c r="B157">
-        <v>7</v>
-      </c>
-      <c r="C157">
-        <v>1</v>
-      </c>
-      <c r="D157">
-        <v>1968</v>
-      </c>
-      <c r="E157">
-        <v>0</v>
-      </c>
-      <c r="F157">
-        <v>1</v>
-      </c>
-      <c r="G157">
-        <v>1</v>
-      </c>
-      <c r="H157">
-        <v>5257.304601</v>
-      </c>
-      <c r="I157">
-        <v>1051.46092</v>
-      </c>
-    </row>
-    <row r="158">
-      <c r="A158" t="inlineStr">
-        <is>
-          <t>CPUE</t>
-        </is>
-      </c>
-      <c r="B158">
-        <v>7</v>
-      </c>
-      <c r="C158">
-        <v>1</v>
-      </c>
-      <c r="D158">
-        <v>1969</v>
-      </c>
-      <c r="E158">
-        <v>0</v>
-      </c>
-      <c r="F158">
-        <v>1</v>
-      </c>
-      <c r="G158">
-        <v>1</v>
-      </c>
-      <c r="H158">
-        <v>6712.468418</v>
-      </c>
-      <c r="I158">
-        <v>1342.493684</v>
-      </c>
-    </row>
-    <row r="159">
-      <c r="A159" t="inlineStr">
-        <is>
-          <t>CPUE</t>
-        </is>
-      </c>
-      <c r="B159">
-        <v>7</v>
-      </c>
-      <c r="C159">
-        <v>1</v>
-      </c>
-      <c r="D159">
-        <v>1970</v>
-      </c>
-      <c r="E159">
-        <v>0</v>
-      </c>
-      <c r="F159">
-        <v>1</v>
-      </c>
-      <c r="G159">
-        <v>1</v>
-      </c>
-      <c r="H159">
-        <v>5679.809828</v>
-      </c>
-      <c r="I159">
-        <v>1135.961966</v>
-      </c>
-    </row>
-    <row r="160">
-      <c r="A160" t="inlineStr">
-        <is>
-          <t>CPUE</t>
-        </is>
-      </c>
-      <c r="B160">
-        <v>7</v>
-      </c>
-      <c r="C160">
-        <v>1</v>
-      </c>
-      <c r="D160">
-        <v>1971</v>
-      </c>
-      <c r="E160">
-        <v>0</v>
-      </c>
-      <c r="F160">
-        <v>1</v>
-      </c>
-      <c r="G160">
-        <v>1</v>
-      </c>
-      <c r="H160">
-        <v>5257.331283</v>
-      </c>
-      <c r="I160">
-        <v>1051.466257</v>
-      </c>
-    </row>
-    <row r="161">
-      <c r="A161" t="inlineStr">
-        <is>
-          <t>CPUE</t>
-        </is>
-      </c>
-      <c r="B161">
-        <v>7</v>
-      </c>
-      <c r="C161">
-        <v>1</v>
-      </c>
-      <c r="D161">
-        <v>1972</v>
-      </c>
-      <c r="E161">
-        <v>0</v>
-      </c>
-      <c r="F161">
-        <v>1</v>
-      </c>
-      <c r="G161">
-        <v>1</v>
-      </c>
-      <c r="H161">
-        <v>5726.743484</v>
-      </c>
-      <c r="I161">
-        <v>1145.348697</v>
-      </c>
-    </row>
-    <row r="162">
-      <c r="A162" t="inlineStr">
-        <is>
-          <t>CPUE</t>
-        </is>
-      </c>
-      <c r="B162">
-        <v>7</v>
-      </c>
-      <c r="C162">
-        <v>1</v>
-      </c>
-      <c r="D162">
-        <v>1973</v>
-      </c>
-      <c r="E162">
-        <v>0</v>
-      </c>
-      <c r="F162">
-        <v>1</v>
-      </c>
-      <c r="G162">
-        <v>1</v>
-      </c>
-      <c r="H162">
-        <v>4787.923949</v>
-      </c>
-      <c r="I162">
-        <v>957.5847898</v>
-      </c>
-    </row>
-    <row r="163">
-      <c r="A163" t="inlineStr">
-        <is>
-          <t>CPUE</t>
-        </is>
-      </c>
-      <c r="B163">
-        <v>7</v>
-      </c>
-      <c r="C163">
-        <v>1</v>
-      </c>
-      <c r="D163">
-        <v>1974</v>
-      </c>
-      <c r="E163">
-        <v>0</v>
-      </c>
-      <c r="F163">
-        <v>1</v>
-      </c>
-      <c r="G163">
-        <v>1</v>
-      </c>
-      <c r="H163">
-        <v>4740.992588</v>
-      </c>
-      <c r="I163">
-        <v>948.1985175999999</v>
-      </c>
-    </row>
-    <row r="164">
-      <c r="A164" t="inlineStr">
-        <is>
-          <t>CPUE</t>
-        </is>
-      </c>
-      <c r="B164">
-        <v>7</v>
-      </c>
-      <c r="C164">
-        <v>1</v>
-      </c>
-      <c r="D164">
-        <v>1975</v>
-      </c>
-      <c r="E164">
-        <v>0</v>
-      </c>
-      <c r="F164">
-        <v>1</v>
-      </c>
-      <c r="G164">
-        <v>1</v>
-      </c>
-      <c r="H164">
-        <v>4271.57446</v>
-      </c>
-      <c r="I164">
-        <v>854.3148919</v>
-      </c>
-    </row>
-    <row r="165">
-      <c r="A165" t="inlineStr">
-        <is>
-          <t>CPUE</t>
-        </is>
-      </c>
-      <c r="B165">
-        <v>7</v>
-      </c>
-      <c r="C165">
-        <v>1</v>
-      </c>
-      <c r="D165">
-        <v>1976</v>
-      </c>
-      <c r="E165">
-        <v>0</v>
-      </c>
-      <c r="F165">
-        <v>1</v>
-      </c>
-      <c r="G165">
-        <v>1</v>
-      </c>
-      <c r="H165">
-        <v>4318.523058</v>
-      </c>
-      <c r="I165">
         <v>863.7046116</v>
       </c>
     </row>

</xml_diff>

<commit_message>
EBS pollock: match ADMB comp/index data encoding + AMAK avgsel; two-stage fit
Composition / index alignment to the ADMB m23_rceattle_full data file and
likelihood:
- BTS/ATS age-comp sample sizes truncated to integer (ADMB reads init_ivector).
- 2020 ATS age-comp sample size set to 1 (ADMB sam_ats; COVID-year survey).
- ATS biomass index Log_sd = sqrt(log(CV^2 + 1)) (ADMB lvarb_ats CV->log-SD).
- AMAK avgsel base-level selectivity penalty enabled (Sel_avgsel_pen = 10).

Fit in two stages (time-varying selectivity off, then on and seeded from the
first) so the model converges from default parameters rather than the weakly
identified population scale running away.

With these and the earlier config edits, the Rceattle objective reproduces the
ADMB reference objective term-by-term to machine precision at the MLE. Header
documents the full ADMB<->Rceattle alignment.
</commit_message>
<xml_diff>
--- a/EBS pollock/Data/2024_EBS_pollock_m23_rceattle_full.xlsx
+++ b/EBS pollock/Data/2024_EBS_pollock_m23_rceattle_full.xlsx
@@ -34489,7 +34489,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AM8"/>
+  <dimension ref="A1:AN8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -34685,6 +34685,11 @@
       </c>
       <c r="AM1" s="1" t="inlineStr">
         <is>
+          <t>Sel_avgsel_pen</t>
+        </is>
+      </c>
+      <c r="AN1" s="1" t="inlineStr">
+        <is>
           <t>Index_loglike</t>
         </is>
       </c>
@@ -34810,6 +34815,9 @@
       <c r="AJ2">
         <v>1</v>
       </c>
+      <c r="AM2">
+        <v>10</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -34932,7 +34940,10 @@
       <c r="AL3">
         <v>2</v>
       </c>
-      <c r="AM3" t="inlineStr">
+      <c r="AM3">
+        <v>10</v>
+      </c>
+      <c r="AN3" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
@@ -35062,7 +35073,7 @@
       <c r="AK4">
         <v>1982</v>
       </c>
-      <c r="AM4" t="inlineStr">
+      <c r="AN4" t="inlineStr">
         <is>
           <t>MVN</t>
         </is>
@@ -35192,6 +35203,9 @@
       <c r="AL5">
         <v>2</v>
       </c>
+      <c r="AM5">
+        <v>10</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -35540,7 +35554,10 @@
       <c r="AJ8">
         <v>1</v>
       </c>
-      <c r="AM8" t="inlineStr">
+      <c r="AM8">
+        <v>10</v>
+      </c>
+      <c r="AN8" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
@@ -37491,7 +37508,7 @@
         <v>3628.9293</v>
       </c>
       <c r="I62">
-        <v>0.1890055559914049</v>
+        <v>0.1873494870789829</v>
       </c>
     </row>
     <row r="63">
@@ -37522,7 +37539,7 @@
         <v>2944.77187</v>
       </c>
       <c r="I63">
-        <v>0.1486974201502407</v>
+        <v>0.1478851611270841</v>
       </c>
     </row>
     <row r="64">
@@ -37553,7 +37570,7 @@
         <v>3590.84054</v>
       </c>
       <c r="I64">
-        <v>0.1353304260066085</v>
+        <v>0.1347168767363003</v>
       </c>
     </row>
     <row r="65">
@@ -37584,7 +37601,7 @@
         <v>4141.37057</v>
       </c>
       <c r="I65">
-        <v>0.2043826592412376</v>
+        <v>0.2022952543293446</v>
       </c>
     </row>
     <row r="66">
@@ -37615,7 +37632,7 @@
         <v>3625.86364</v>
       </c>
       <c r="I66">
-        <v>0.128670997125529</v>
+        <v>0.1281431441630527</v>
       </c>
     </row>
     <row r="67">
@@ -37646,7 +37663,7 @@
         <v>4305.86229</v>
       </c>
       <c r="I67">
-        <v>0.1244069675066176</v>
+        <v>0.1239295968627708</v>
       </c>
     </row>
     <row r="68">
@@ -37677,7 +37694,7 @@
         <v>4009.93704</v>
       </c>
       <c r="I68">
-        <v>0.1444254097316201</v>
+        <v>0.1436806697877727</v>
       </c>
     </row>
     <row r="69">
@@ -37708,7 +37725,7 @@
         <v>1872.86327</v>
       </c>
       <c r="I69">
-        <v>0.1565715739622573</v>
+        <v>0.155624534826529</v>
       </c>
     </row>
     <row r="70">
@@ -37739,7 +37756,7 @@
         <v>2277.944</v>
       </c>
       <c r="I70">
-        <v>0.1754534571525903</v>
+        <v>0.1741252305022351</v>
       </c>
     </row>
     <row r="71">
@@ -37770,7 +37787,7 @@
         <v>1405.59025</v>
       </c>
       <c r="I71">
-        <v>0.2603814945358365</v>
+        <v>0.2561231609619358</v>
       </c>
     </row>
     <row r="72">
@@ -37801,7 +37818,7 @@
         <v>1324.78137</v>
       </c>
       <c r="I72">
-        <v>0.3209667116620156</v>
+        <v>0.3131318205262479</v>
       </c>
     </row>
     <row r="73">
@@ -37832,7 +37849,7 @@
         <v>2642.6749</v>
       </c>
       <c r="I73">
-        <v>0.250335612602216</v>
+        <v>0.246541377220169</v>
       </c>
     </row>
     <row r="74">
@@ -37863,7 +37880,7 @@
         <v>2295.95185</v>
       </c>
       <c r="I74">
-        <v>0.1591845839449987</v>
+        <v>0.1581897698952716</v>
       </c>
     </row>
     <row r="75">
@@ -37894,7 +37911,7 @@
         <v>4729.82772</v>
       </c>
       <c r="I75">
-        <v>0.1610945778803123</v>
+        <v>0.1600638579876487</v>
       </c>
     </row>
     <row r="76">
@@ -37925,7 +37942,7 @@
         <v>4828.79348</v>
       </c>
       <c r="I76">
-        <v>0.08740508198333634</v>
+        <v>0.08723883323368406</v>
       </c>
     </row>
     <row r="77">
@@ -37956,7 +37973,7 @@
         <v>2499.40106</v>
       </c>
       <c r="I77">
-        <v>0.1843558992489185</v>
+        <v>0.1828176628598207</v>
       </c>
     </row>
     <row r="78">
@@ -37987,7 +38004,7 @@
         <v>3617</v>
       </c>
       <c r="I78">
-        <v>0.4493864860381532</v>
+        <v>0.428886642193354</v>
       </c>
     </row>
     <row r="79">
@@ -38018,7 +38035,7 @@
         <v>3834.04251</v>
       </c>
       <c r="I79">
-        <v>0.3203175099902583</v>
+        <v>0.3125284413146217</v>
       </c>
     </row>
     <row r="80">
@@ -38049,7 +38066,7 @@
         <v>2870.636995</v>
       </c>
       <c r="I80">
-        <v>0.2628487802234291</v>
+        <v>0.2584711475575581</v>
       </c>
     </row>
     <row r="81">
@@ -47257,7 +47274,7 @@
         <v>1982</v>
       </c>
       <c r="H62">
-        <v>162.0393239</v>
+        <v>162</v>
       </c>
       <c r="I62">
         <v>10950974.45</v>
@@ -47330,7 +47347,7 @@
         <v>1983</v>
       </c>
       <c r="H63">
-        <v>130.7006627</v>
+        <v>130</v>
       </c>
       <c r="I63">
         <v>45353039.8</v>
@@ -47403,7 +47420,7 @@
         <v>1984</v>
       </c>
       <c r="H64">
-        <v>63.27312528</v>
+        <v>63</v>
       </c>
       <c r="I64">
         <v>4810111.378</v>
@@ -47476,7 +47493,7 @@
         <v>1985</v>
       </c>
       <c r="H65">
-        <v>73.53570806</v>
+        <v>73</v>
       </c>
       <c r="I65">
         <v>49329672.64</v>
@@ -47549,7 +47566,7 @@
         <v>1986</v>
       </c>
       <c r="H66">
-        <v>151.9481692</v>
+        <v>151</v>
       </c>
       <c r="I66">
         <v>29490315.26</v>
@@ -47622,7 +47639,7 @@
         <v>1987</v>
       </c>
       <c r="H67">
-        <v>61.21469951</v>
+        <v>61</v>
       </c>
       <c r="I67">
         <v>4901555.37</v>
@@ -47695,7 +47712,7 @@
         <v>1988</v>
       </c>
       <c r="H68">
-        <v>82.23254369999999</v>
+        <v>82</v>
       </c>
       <c r="I68">
         <v>15721198.77</v>
@@ -47768,7 +47785,7 @@
         <v>1989</v>
       </c>
       <c r="H69">
-        <v>53.19136982</v>
+        <v>53</v>
       </c>
       <c r="I69">
         <v>9045388.605</v>
@@ -47841,7 +47858,7 @@
         <v>1990</v>
       </c>
       <c r="H70">
-        <v>48.26632231</v>
+        <v>48</v>
       </c>
       <c r="I70">
         <v>22226901.34</v>
@@ -47914,7 +47931,7 @@
         <v>1991</v>
       </c>
       <c r="H71">
-        <v>79.42427175</v>
+        <v>79</v>
       </c>
       <c r="I71">
         <v>32298906.47</v>
@@ -47987,7 +48004,7 @@
         <v>1992</v>
       </c>
       <c r="H72">
-        <v>85.22046362</v>
+        <v>85</v>
       </c>
       <c r="I72">
         <v>15591259.43</v>
@@ -48060,7 +48077,7 @@
         <v>1993</v>
       </c>
       <c r="H73">
-        <v>91.98361398</v>
+        <v>91</v>
       </c>
       <c r="I73">
         <v>26831974.61</v>
@@ -48133,7 +48150,7 @@
         <v>1994</v>
       </c>
       <c r="H74">
-        <v>86.85138402</v>
+        <v>86</v>
       </c>
       <c r="I74">
         <v>16300489.78</v>
@@ -48206,7 +48223,7 @@
         <v>1995</v>
       </c>
       <c r="H75">
-        <v>104.8977063</v>
+        <v>104</v>
       </c>
       <c r="I75">
         <v>16172066.37</v>
@@ -48279,7 +48296,7 @@
         <v>1996</v>
       </c>
       <c r="H76">
-        <v>226.4696079</v>
+        <v>226</v>
       </c>
       <c r="I76">
         <v>19509804.11</v>
@@ -48352,7 +48369,7 @@
         <v>1997</v>
       </c>
       <c r="H77">
-        <v>73.38480423999999</v>
+        <v>73</v>
       </c>
       <c r="I77">
         <v>23321877.34</v>
@@ -48425,7 +48442,7 @@
         <v>1998</v>
       </c>
       <c r="H78">
-        <v>65.18831014</v>
+        <v>65</v>
       </c>
       <c r="I78">
         <v>8710506.469000001</v>
@@ -48498,7 +48515,7 @@
         <v>1999</v>
       </c>
       <c r="H79">
-        <v>95.42897041000001</v>
+        <v>95</v>
       </c>
       <c r="I79">
         <v>9913042.828</v>
@@ -48571,7 +48588,7 @@
         <v>2000</v>
       </c>
       <c r="H80">
-        <v>90.69342702</v>
+        <v>90</v>
       </c>
       <c r="I80">
         <v>10448664.91</v>
@@ -48644,7 +48661,7 @@
         <v>2001</v>
       </c>
       <c r="H81">
-        <v>183.0103987</v>
+        <v>183</v>
       </c>
       <c r="I81">
         <v>19866054.3</v>
@@ -48717,7 +48734,7 @@
         <v>2002</v>
       </c>
       <c r="H82">
-        <v>186.3252567</v>
+        <v>186</v>
       </c>
       <c r="I82">
         <v>13635855.02</v>
@@ -48790,7 +48807,7 @@
         <v>2003</v>
       </c>
       <c r="H83">
-        <v>125.6594543</v>
+        <v>125</v>
       </c>
       <c r="I83">
         <v>5737576.96</v>
@@ -48863,7 +48880,7 @@
         <v>2004</v>
       </c>
       <c r="H84">
-        <v>188.6575824</v>
+        <v>188</v>
       </c>
       <c r="I84">
         <v>3971309.628</v>
@@ -48936,7 +48953,7 @@
         <v>2005</v>
       </c>
       <c r="H85">
-        <v>194.4902529</v>
+        <v>194</v>
       </c>
       <c r="I85">
         <v>4008208.162</v>
@@ -49009,7 +49026,7 @@
         <v>2006</v>
       </c>
       <c r="H86">
-        <v>329.6148551</v>
+        <v>329</v>
       </c>
       <c r="I86">
         <v>8156013.515</v>
@@ -49082,7 +49099,7 @@
         <v>2007</v>
       </c>
       <c r="H87">
-        <v>192.6952151</v>
+        <v>192</v>
       </c>
       <c r="I87">
         <v>27341965.7</v>
@@ -49155,7 +49172,7 @@
         <v>2008</v>
       </c>
       <c r="H88">
-        <v>235.4060181</v>
+        <v>235</v>
       </c>
       <c r="I88">
         <v>5026908.871</v>
@@ -49228,7 +49245,7 @@
         <v>2009</v>
       </c>
       <c r="H89">
-        <v>144.7225262</v>
+        <v>144</v>
       </c>
       <c r="I89">
         <v>8423248.112</v>
@@ -49301,7 +49318,7 @@
         <v>2010</v>
       </c>
       <c r="H90">
-        <v>107.8894407</v>
+        <v>107</v>
       </c>
       <c r="I90">
         <v>4800589.205</v>
@@ -49374,7 +49391,7 @@
         <v>2011</v>
       </c>
       <c r="H91">
-        <v>165.2688663</v>
+        <v>165</v>
       </c>
       <c r="I91">
         <v>12920051.51</v>
@@ -49447,7 +49464,7 @@
         <v>2012</v>
       </c>
       <c r="H92">
-        <v>107.1237964</v>
+        <v>107</v>
       </c>
       <c r="I92">
         <v>12972591.79</v>
@@ -49520,7 +49537,7 @@
         <v>2013</v>
       </c>
       <c r="H93">
-        <v>66.52654145</v>
+        <v>66</v>
       </c>
       <c r="I93">
         <v>12516351.14</v>
@@ -49593,7 +49610,7 @@
         <v>2014</v>
       </c>
       <c r="H94">
-        <v>117.6641689</v>
+        <v>117</v>
       </c>
       <c r="I94">
         <v>25378686.14</v>
@@ -49666,7 +49683,7 @@
         <v>2015</v>
       </c>
       <c r="H95">
-        <v>103.6700104</v>
+        <v>103</v>
       </c>
       <c r="I95">
         <v>14570602.84</v>
@@ -49739,7 +49756,7 @@
         <v>2016</v>
       </c>
       <c r="H96">
-        <v>122.8399641</v>
+        <v>122</v>
       </c>
       <c r="I96">
         <v>7941441.528</v>
@@ -49812,7 +49829,7 @@
         <v>2017</v>
       </c>
       <c r="H97">
-        <v>234.588978</v>
+        <v>234</v>
       </c>
       <c r="I97">
         <v>7835995.184</v>
@@ -49885,7 +49902,7 @@
         <v>2018</v>
       </c>
       <c r="H98">
-        <v>158.3203367</v>
+        <v>158</v>
       </c>
       <c r="I98">
         <v>11286192.27</v>
@@ -49958,7 +49975,7 @@
         <v>2019</v>
       </c>
       <c r="H99">
-        <v>120.6785752</v>
+        <v>120</v>
       </c>
       <c r="I99">
         <v>26795702.01</v>
@@ -50031,7 +50048,7 @@
         <v>2021</v>
       </c>
       <c r="H100">
-        <v>149.479296</v>
+        <v>149</v>
       </c>
       <c r="I100">
         <v>10321941.11</v>
@@ -50104,7 +50121,7 @@
         <v>2022</v>
       </c>
       <c r="H101">
-        <v>172.8341002</v>
+        <v>172</v>
       </c>
       <c r="I101">
         <v>8119155.479</v>
@@ -50177,7 +50194,7 @@
         <v>2023</v>
       </c>
       <c r="H102">
-        <v>126.7773094</v>
+        <v>126</v>
       </c>
       <c r="I102">
         <v>11137835.36</v>
@@ -50250,7 +50267,7 @@
         <v>2024</v>
       </c>
       <c r="H103">
-        <v>64.21408227000001</v>
+        <v>64</v>
       </c>
       <c r="I103">
         <v>16262095.59</v>
@@ -51491,7 +51508,7 @@
         <v>2020</v>
       </c>
       <c r="H120">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I120">
         <v>0</v>

</xml_diff>

<commit_message>
EBS pollock: string switch aliases, condensed comments, rename workflow scripts
- Use string switch aliases instead of integer codes across the scripts:
  Fleet_type 2/0 -> "Survey"/"Off", Catchability "1"/"3" -> "Estimated"/
  "Analytical", Estimate_index_sd 0 -> "Fixed" (data.R, bridging.R, mse.R).
  Regenerated the model xlsx so its switch columns store the aliases too; the
  base two-stage fit is bit-identical (713.6765), so the ADMB match is unchanged.
- Condense verbose comments (data.R ADMB-bridge header ~70 -> ~22 lines; the
  comparison script's two-stage / 2D AR1 / comparison blocks; workflow headers).
- Rename the assessment-workflow scripts 2025 -> 2024 to match the vintage naming
  and fix their internal cross-references.

estDynamics stays numeric (read numerically before conversion); deprecated column
NAMES (Q_index etc.) are unchanged -- data.R runs on main, which keeps them.
</commit_message>
<xml_diff>
--- a/EBS pollock/Data/2024_EBS_pollock_m23_rceattle_full.xlsx
+++ b/EBS pollock/Data/2024_EBS_pollock_m23_rceattle_full.xlsx
@@ -34767,8 +34767,10 @@
       <c r="U2">
         <v>0</v>
       </c>
-      <c r="V2">
-        <v>0</v>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="W2">
         <v>1</v>
@@ -34889,8 +34891,10 @@
       <c r="U3">
         <v>0</v>
       </c>
-      <c r="V3">
-        <v>0</v>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
       </c>
       <c r="W3">
         <v>1</v>
@@ -35022,8 +35026,10 @@
       <c r="U4">
         <v>0</v>
       </c>
-      <c r="V4">
-        <v>0</v>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="W4">
         <v>1</v>
@@ -35132,7 +35138,7 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Estimated</t>
         </is>
       </c>
       <c r="R5">
@@ -35149,8 +35155,10 @@
       <c r="U5">
         <v>0</v>
       </c>
-      <c r="V5">
-        <v>0</v>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="W5">
         <v>1</v>
@@ -35218,7 +35226,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Off</t>
         </is>
       </c>
       <c r="D6">
@@ -35260,7 +35268,7 @@
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>Analytical</t>
         </is>
       </c>
       <c r="R6">
@@ -35277,8 +35285,10 @@
       <c r="U6">
         <v>0</v>
       </c>
-      <c r="V6">
-        <v>0</v>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="W6">
         <v>1</v>
@@ -35334,7 +35344,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>Survey</t>
         </is>
       </c>
       <c r="D7">
@@ -35376,7 +35386,7 @@
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>Analytical</t>
         </is>
       </c>
       <c r="R7">
@@ -35393,8 +35403,10 @@
       <c r="U7">
         <v>0</v>
       </c>
-      <c r="V7">
-        <v>0</v>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="W7">
         <v>1</v>
@@ -35495,7 +35507,7 @@
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Estimated</t>
         </is>
       </c>
       <c r="R8">
@@ -35512,8 +35524,10 @@
       <c r="U8">
         <v>0</v>
       </c>
-      <c r="V8">
-        <v>0</v>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
       </c>
       <c r="W8">
         <v>1</v>

</xml_diff>

<commit_message>
EBS pollock: fix Estimate_index_sd string-alias regression
Converting Estimate_index_sd to "Fixed" for only the AVO/CPUE fleets coerced the
numeric column to character and left "0" strings on the other fleets. Lenient
(main) validators accept "0"; the strict dev-line validator (dev-data-workflow /
perf-profiling, which auto-upgrades column names) rejects it, so the model would
not build there. Set the whole Estimate_index_sd column as a string alias instead.

Regenerated the xlsx; base two-stage fit still bit-identical (713.6765) on main,
and the model now builds on perf-profiling too.
</commit_message>
<xml_diff>
--- a/EBS pollock/Data/2024_EBS_pollock_m23_rceattle_full.xlsx
+++ b/EBS pollock/Data/2024_EBS_pollock_m23_rceattle_full.xlsx
@@ -34769,7 +34769,7 @@
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="W2">
@@ -35028,7 +35028,7 @@
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="W4">
@@ -35157,7 +35157,7 @@
       </c>
       <c r="V5" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="W5">
@@ -35287,7 +35287,7 @@
       </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="W6">
@@ -35405,7 +35405,7 @@
       </c>
       <c r="V7" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="W7">

</xml_diff>